<commit_message>
updated functionality to only keep 3 sentences for the summary and to control cut off points for the body based on patterns in the html page format and footers
</commit_message>
<xml_diff>
--- a/scraped_natural_refrigerants_news.xlsx
+++ b/scraped_natural_refrigerants_news.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,406 +458,783 @@
           <t>attachmenturl</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ATMO Europe: European Private Equity Firm Triton Partners Positions Data Center Cooling as a High-Value Product Segment</t>
+          <t>ATMO Europe: Pascal Outlines Low-Pressure Solid-State Barocaloric Refrigeration Potential</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>European private equity firm Triton has emphasized the rising strategic importance of HVAC&amp;R companies developing data center cooling product portfolios as global demand for data processing and digital infrastructure continues to accelerate. “The growth of data centers in the world is just phenomenal, and the need for cooling is going to be unbelievable, particularly clean cooling,” said Ted Amyuni, Senior Industry Expert at Triton Partners. “It’s a good time to have a product category for data centers.” Amyuni delivered these remarks during the investor panel at the ATMO Europe 2025 Summit. He was joined by Friedrich Ysenburg, Investment Professional at Triton Partners; Timo Kivilaht, Senior Vice President of Global Sales and Solutions at heat exchanger manufacturer Kelvion; and Nicolo Freyberg, Managing Director of bluu unit, a contractor alliance focused on natural refrigerants. Both Kelvion and bluu unit are part of Triton’s HVAC&amp;R investment portfolio. During the panel, participants also underscored the need to build technical capacity to support the transition to natural refrigerants – a core priority for Triton – and the growing investment risks linked to PFAS (per- and polyfluoroalkyl substances). ATMO Europe 2025 took place November 24–25 in Padova, Italy, and was organized by ATMOsphere, publisher of NaturalRefrigerants.com. Triton – a firm with more than 45 portfolio companies and a combined turnover of more than €18 billion ($20.8 billion) – was the event’s platinum sponsor. “The growth of data centers in the world is just phenomenal, and the need for cooling is going to be unbelievable, particularly clean cooling. It’s a good time to have a product category for data centers.” Ted Amyuni, Senior Industry Expert at Triton Partners Data centers Commercial HVAC equipment manufacturer FläktGroup – which Triton recently sold to Samsung – was highlighted by Amyuni as a clear example of the value embedded in data center cooling. When Triton purchased FläktGroup, the company had no offerings for data center applications and was concentrated almost entirely on indoor climate solutions, which accounted for roughly 80% of its business, he noted. By the time Triton exited, data center solutions had grown to about 25% of the company’s portfolio. “We started a data center vertical from the ground up, adding big value to FläktGroup,” Amyuni said. “Samsung wanted to acquire FläktGroup to get into commercial HVAC and, most importantly, data centers. That exit was very successful.” “We do a lot of research to really understand the opportunities,” added Ysenburg. “You need to differentiate yourself and talk about value creation in terms of really how we are going to improve companies. [Our companies] are very successful because we’ve been early on investing in [the sustainable cooling] space, when many others didn’t see it.” In August, Triton sold a majority stake in Kelvion to U.S. private equity firm Apollo, maintaining a minority interest in the manufacturer. Kelvion has placed an increased focus on data center cooling solutions in recent years, which have become the company’s largest and fastest-growing segment, accounting for 50% of its €1.6 billion ($1.85 billion) order intake in 2024, according to Kivilaht. “Data centers are clearly one of the biggest growth drivers over the last eight years, and [this trend] is going to continue over the next couple of years with a lot of investments,” Kivilaht noted. In addition to the development of larger data centers, solutions will also be needed for existing facilities that will have to be upgraded and expanded over the coming years to meet demand. To prepare for the future, Kivilaht said, Kelvion has expanded its production sites in the U.S. It is also building an R&amp;D center in the U.K. that is focused on the development and testing of new cooling solutions for data centers. “We can actually test whatever kind of equipment is going into a data center to really figure out what’s going to be the right cooling solution,” he explained. Amyuni noted a growing trend of large companies acquiring smaller firms and startups that specialize in liquid cooling technologies for data centers, something that was not as common a few years ago. “Data centers are clearly one of the biggest growth drivers over the last eight years, and [this trend] is going to continue over the next couple of years with a lot of investments.” Timo Kivilaht, Senior Vice President of Global Sales and Solutions at Kelvion Building technical capacity Another major theme of the investor panel was the urgent need to expand technical capacity across Europe to support the shift toward natural refrigerants, particularly with regulatory tailwinds helping to drive the transition. Bluu unit was founded by Triton in 2023 following their acquisition of a majority stake in Germany-based Kälte Eckert Group, with the aim of creating a leading alliance of HVAC&amp;R contractors for natural refrigerant-based projects in Europe. “When we started, the market was in a very different position than it’s today,” Freyberg explained. “The EU F-gas Regulation was just about to be run through the EU legislation, and PFAS was known but not as apparent as today. There was clear potential, and we believe the market potential is so big.” “We have a lot of good competitors in the technical building market, but no one is as focused on natural refrigerants,” he added. “When companies join bluu unit, they are not 100% natural refrigerants yet, but they need to have the clear understanding that this is the way forward – that’s where the market is going.” Since its inception, bluu unit has entered the Swiss market and now consists of more than 27 contractors that collectively employ more than 900 people. In addition to its Swiss expansion, the alliance eventually plans to expand outside Germany, Switzerland and Austria. Over the last two years, Bluu unit has generated over €240 million ($278 million) in sales and completed more than 10,000 projects, according to Freyberg. Core parts of bluu unit’s work are training, knowledge transfer and collaboration. “We train with our suppliers as a group,” he noted. “We invite other companies that are not that advanced [in natural refrigerants] to send their people to work together on projects to help get them equipped with the right skillset.” “When companies join bluu unit, they are not 100% natural refrigerants yet, but they need to have the clear understanding that this is the way forward – that’s where the market is going.” Nicolo Freyberg, Managing Director of bluu unit PFAS PFAS regulation is another major trend that Triton is monitoring closely, both as a potential investment risk and as a catalyst for innovation, explained Ysenburg. “When things change – like when PFAS regulation comes into place – there’s a lot of capital needed to foster that change,” he noted. “On the risk-management side, we have PFAS audits where we look into the exposure of our companies and try to handle that.” Freyberg echoed the view that PFAS restrictions, while challenging, are also creating significant market opportunities. However, he stressed the importance of pacing the transition. “Everyone has a clear state of mind about the impact [of PFAS], and, in the long term, I only see it as an opportunity for us that creates market growth and change,” he said. “But we need to find a balance here of not moving too quickly because you might lose people that are still quite overwhelmed by natural refrigerants.” Kivilaht pointed to developments in China as further evidence of how rapidly PFAS-related changes may unfold, noting that China’s HVAC&amp;R sector is already moving quickly on PFAS compliance. In his view both China and Europe are positioned to move far ahead of other regions, including the U.S. and Asia–Pacific, in adapting to PFAS regulations and advancing cleaner cooling technologies. “Everyone has a clear state of mind about the impact [of PFAS], and, in the long term, I only see it as an opportunity for us that creates market growth and change.” Nicolo Freyberg, Managing Director of bluu unit</t>
+          <t>Adam Slavney, CEO and Co-Founder of U.S.-based startup Pascal, outlined the potential of the company’s low-pressure solid-state barocaloric refrigeration design at the ATMOsphere (ATMO) Europe Summit 2025.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45992</v>
+        <v>46048</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>European private equity firm Triton has emphasized the rising strategic importance of HVAC&amp;R companies developing data center cooling product portfolios as global demand for data processing and digital infrastructure continues to accelerate. “The growth of data centers in the world is just phenomenal, and the need for cooling is going to be unbelievable, particularly clean cooling,” said Ted Amyuni, Senior Industry Expert at Triton Partners. “It’s a good time to have a product category for data centers.” Amyuni delivered these remarks during the investor panel at the ATMO Europe 2025 Summit. He was joined by Friedrich Ysenburg, Investment Professional at Triton Partners; Timo Kivilaht, Senior Vice President of Global Sales and Solutions at heat exchanger manufacturer Kelvion; and Nicolo Freyberg, Managing Director of bluu unit, a contractor alliance focused on natural refrigerants. Both Kelvion and bluu unit are part of Triton’s HVAC&amp;R investment portfolio. During the panel, participants also underscored the need to build technical capacity to support the transition to natural refrigerants – a core priority for Triton – and the growing investment risks linked to PFAS (per- and polyfluoroalkyl substances). ATMO Europe 2025 took place November 24–25 in Padova, Italy, and was organized by ATMOsphere, publisher of NaturalRefrigerants.com. Triton – a firm with more than 45 portfolio companies and a combined turnover of more than €18 billion ($20.8 billion) – was the event’s platinum sponsor. “The growth of data centers in the world is just phenomenal, and the need for cooling is going to be unbelievable, particularly clean cooling. It’s a good time to have a product category for data centers.” Ted Amyuni, Senior Industry Expert at Triton Partners Data centers Commercial HVAC equipment manufacturer FläktGroup – which Triton recently sold to Samsung – was highlighted by Amyuni as a clear example of the value embedded in data center cooling. When Triton purchased FläktGroup, the company had no offerings for data center applications and was concentrated almost entirely on indoor climate solutions, which accounted for roughly 80% of its business, he noted. By the time Triton exited, data center solutions had grown to about 25% of the company’s portfolio. “We started a data center vertical from the ground up, adding big value to FläktGroup,” Amyuni said. “Samsung wanted to acquire FläktGroup to get into commercial HVAC and, most importantly, data centers. That exit was very successful.” “We do a lot of research to really understand the opportunities,” added Ysenburg. “You need to differentiate yourself and talk about value creation in terms of really how we are going to improve companies. [Our companies] are very successful because we’ve been early on investing in [the sustainable cooling] space, when many others didn’t see it.” In August, Triton sold a majority stake in Kelvion to U.S. private equity firm Apollo, maintaining a minority interest in the manufacturer. Kelvion has placed an increased focus on data center cooling solutions in recent years, which have become the company’s largest and fastest-growing segment, accounting for 50% of its €1.6 billion ($1.85 billion) order intake in 2024, according to Kivilaht. “Data centers are clearly one of the biggest growth drivers over the last eight years, and [this trend] is going to continue over the next couple of years with a lot of investments,” Kivilaht noted. In addition to the development of larger data centers, solutions will also be needed for existing facilities that will have to be upgraded and expanded over the coming years to meet demand. To prepare for the future, Kivilaht said, Kelvion has expanded its production sites in the U.S. It is also building an R&amp;D center in the U.K. that is focused on the development and testing of new cooling solutions for data centers. “We can actually test whatever kind of equipment is going into a data center to really figure out what’s going to be the right cooling solution,” he explained. Amyuni noted a growing trend of large companies acquiring smaller firms and startups that specialize in liquid cooling technologies for data centers, something that was not as common a few years ago. “Data centers are clearly one of the biggest growth drivers over the last eight years, and [this trend] is going to continue over the next couple of years with a lot of investments.” Timo Kivilaht, Senior Vice President of Global Sales and Solutions at Kelvion Building technical capacity Another major theme of the investor panel was the urgent need to expand technical capacity across Europe to support the shift toward natural refrigerants, particularly with regulatory tailwinds helping to drive the transition. Bluu unit was founded by Triton in 2023 following their acquisition of a majority stake in Germany-based Kälte Eckert Group, with the aim of creating a leading alliance of HVAC&amp;R contractors for natural refrigerant-based projects in Europe. “When we started, the market was in a very different position than it’s today,” Freyberg explained. “The EU F-gas Regulation was just about to be run through the EU legislation, and PFAS was known but not as apparent as today. There was clear potential, and we believe the market potential is so big.” “We have a lot of good competitors in the technical building market, but no one is as focused on natural refrigerants,” he added. “When companies join bluu unit, they are not 100% natural refrigerants yet, but they need to have the clear understanding that this is the way forward – that’s where the market is going.” Since its inception, bluu unit has entered the Swiss market and now consists of more than 27 contractors that collectively employ more than 900 people. In addition to its Swiss expansion, the alliance eventually plans to expand outside Germany, Switzerland and Austria. Over the last two years, Bluu unit has generated over €240 million ($278 million) in sales and completed more than 10,000 projects, according to Freyberg. Core parts of bluu unit’s work are training, knowledge transfer and collaboration. “We train with our suppliers as a group,” he noted. “We invite other companies that are not that advanced [in natural refrigerants] to send their people to work together on projects to help get them equipped with the right skillset.” “When companies join bluu unit, they are not 100% natural refrigerants yet, but they need to have the clear understanding that this is the way forward – that’s where the market is going.” Nicolo Freyberg, Managing Director of bluu unit PFAS PFAS regulation is another major trend that Triton is monitoring closely, both as a potential investment risk and as a catalyst for innovation, explained Ysenburg. “When things change – like when PFAS regulation comes into place – there’s a lot of capital needed to foster that change,” he noted. “On the risk-management side, we have PFAS audits where we look into the exposure of our companies and try to handle that.” Freyberg echoed the view that PFAS restrictions, while challenging, are also creating significant market opportunities. However, he stressed the importance of pacing the transition. “Everyone has a clear state of mind about the impact [of PFAS], and, in the long term, I only see it as an opportunity for us that creates market growth and change,” he said. “But we need to find a balance here of not moving too quickly because you might lose people that are still quite overwhelmed by natural refrigerants.” Kivilaht pointed to developments in China as further evidence of how rapidly PFAS-related changes may unfold, noting that China’s HVAC&amp;R sector is already moving quickly on PFAS compliance. In his view both China and Europe are positioned to move far ahead of other regions, including the U.S. and Asia–Pacific, in adapting to PFAS regulations and advancing cleaner cooling technologies. “Everyone has a clear state of mind about the impact [of PFAS], and, in the long term, I only see it as an opportunity for us that creates market growth and change.” Nicolo Freyberg, Managing Director of bluu unit</t>
+          <t>Adam Slavney, CEO and Co-Founder of U.S.-based startup Pascal, outlined the potential of the company’s low-pressure solid-state barocaloric refrigeration design at the ATMOsphere (ATMO) Europe Summit 2025.
+In a presentation, Slavney shared details about the technology, costs and efficiency. The event, organized by ATMOSphere, was held November 24–25 in Padua, Italy. ATMOsphere is the publisher of NaturalRefrigerants.com.
+“When the solid undergoes a phase transition between ordered and disordered states under applied pressure, there is a very large change in entropy,” Slavney said. “It absorbs or releases heat, with Pascal’s materials producing a temperature change of more than 30°C [54°F] in a single pressurization stage.”
+The technology: The system cycles through pressurizing two thin–tubed heat exchangers packed with Pascal’s solid powder material, with one heat exchanger hot at any given time and the other cold.
+“We use a gas compressor, preferably a CO2 one, to apply up to 20bar [290psi] pressure to the solid refrigerant material,” Slavney said, with the on/off cycle lasting from as few as 30 seconds up to several minutes. “We’ve observed a temperature range from −10 to 50°C [14 to 122°F] on the surface of the tube,” he added.
+For refrigeration, a secondary heat transfer fluid circulates to absorb heat from the barocaloric solid, transferring it to the ambient air and carrying cooling to the refrigerated space.
+The startup, founded in 2023 as a spin–out of a Harvard chemistry lab, raised venture funding to develop the technology from Khosla Ventures and The Engine Ventures.
+Costs/efficiency: “We can build the system using roughly 80% off-the-shelf components,” Slavney said, which supports cost parity with existing refrigeration technology.
+The company needs a CO2 compressor capable of operating at 10‒20bar (145‒290psi) and a thin-walled heat exchanger to increase efficiency, according to Slavney. “If you produce compressors or heat exchangers and are interested in pushing the envelope, I want to talk to you,” he added.
+He compared Pascal’s solid refrigerant system to a propane (R290) gas compression system. Every mole of propane produces 14kJ of energy per cycle, while sending a mole of CO2 over a similar pressure range produces 26kJ of energy per cycle in the solid–state system.
+However, Pascal’s system incurs additional losses, including heating and cooling of the heat exchangers. “We think we will net out ahead,” Slavney said. “By the end of 2026, we hope to demonstrate a 20% energy efficiency improvement over a state-of-the-art compression system.”
+Product development: Pascal has built an integrated barocaloric benchtop system capable of 0.03–0.04kW (.009‒.01TR) of cooling power using air as the secondary heat-transfer fluid, according to Slaveny. In approximately 90 minutes, it lowers the ambient temperature to a 3°C (37°F) refrigeration temperature.
+The company planned to move the benchtop into a commercial demonstration with controlled insulation boundaries by the end of 2025.
+Although its customers are driving commercial development, Slavney noted, larger applications, such as commercial HVAC, would provide better economies of scale in terms of efficiency.
+Quotable: “Traditionally, calorics have suffered from very high operating pressures, which leads to thick metal walls and expensive components,” Slavney said. “Pascal was founded on driving down the pressure, and now our systems operate in a conventional HVAC range.”
+“Pascal’s materials produce a temperature change of more than 30°C [54°F] in a single pressurization stage.”
+Adam Slavney, CEO and Co-Founder of Pascal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-european-private-equity-firm-triton-partners-positions-data-center-cooling-as-a-high-value-product-segment/</t>
+          <t>https://naturalrefrigerants.com/news/atmo-europe-pascal-outlines-low-pressure-solid-state-barocaloric-refrigeration-potential/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SWEP Heat Exchangers Integral Part of New CO2-Based Cooling System at CERN</t>
+          <t>ATMOsphere Releases ‘Clean Cooling for Data Centers 2025,’ a New Report Featuring Interviews With 9 Cooling System and Component Manufacturers</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>In collaboration with CERN, Swedish-based manufacturer SWEP is supplying brazed plate heat exchangers (BPHE) for the laboratory’s new CO2 (R744)-based cooling system, which includes its Q185H model developed specifically for the project. CERN is updating its ATLAS and CMS sites at the Large Hadron Collider (LHC), located on the France–Switzerland border, in preparation for its fourth operational run, scheduled to begin in 2030. The renovation includes the installation of two new CO2 systems capable of cooling the refrigerant down to −53°C (−63.4°F). To regulate the temperature of the particle detectors in CERN’s new High-Luminosity LHC program, SWEP engineers adapted the company’s B185 BPHE to include a Q-pipe. The newly created Q185H heat exchanger will act as a CO2 evaporator to absorb and remove the increased thermal load resulting from higher radiation levels, according to SWEP. “The entire installation was dimensioned and built specifically to incorporate [our] robust units,” SWEP said. Both its B185 and Q185H BPHEs will “play critical roles” in the cooling system, acting as CO2 superheaters ‒ preventing liquid droplets from entering and damaging compressors ‒ and as CO2 cascades, building a thermal bridge between stages, the company added. The previous refrigeration systems at the ATLAS and CMS sites used synthetic high-GWP-based refrigerants. The new CO2 system is expected to reduce the facility’s greenhouse gas emissions by 40,000 metric tons of CO2e per year, according to CERN. CO2 system details: The combined 1.3MW (370TR) cooling system features 18 modules, seven installed at ATLAS and 11 at CMS, each supplying 70kW (20TR) of capacity.  Due to the lack of space around the detectors, the cooling system, positioned on the surface, will pipe the −53°C CO2 refrigerant 90m (295ft) underground to the heat exchangers. “The unique properties of CO2 enable the use of small pipes ‒ a significant advantage where space is limited,” SWEP said. The cooling systems represent a novel combination of subcritical and transcritical CO2 technologies, said Dirk Leuteritz, Head of Sales at Compact Kältetechnik ‒ the German company that helped develop the solution.  CO2 evaporator: With a vertical tube for rising vapor and a separate tube for descending condensate, the Q185H heat exchanger will maintain the temperature of the detectors below −25°C (−13°F), as required.  The design passively transfers heat, with high temperatures from the radiation detector boiling a two–phase liquid fluid, like helium or nitrogen. The resulting vapor rises through the Q-pipe to the upper end of the BPHE, where the −53°C CO2 refrigerant rejects the heat. Gravity pulls the condensed liquid back into contact with the heat from the detector, restarting the evaporation cycle.  Moving the market: In 2005 SWEP developed its first high-pressure CO2 heat exchanger for CERN’s LHC beauty, or bottom quark, experiment using CO2 cooling.  As a result of the collaboration, SWEP introduced its reinforced B16DW CO2 heat exchanger to the refrigeration market.  Quotable: “We [have] pushed the boundaries of what can be achieved with CO2 natural refrigerant,“ said Yann Herpin, Cooling Engineer at CERN. “We are proud to say that this new system is paving the way for further developments in CO2 refrigeration technology, which will lead to reduced emissions in many other industrial applications.” “We are proud to say that this new system is paving the way for further developments in CO2 refrigeration technology.” Yann Herpin, Cooling Engineer at CERN</t>
+          <t>ATMOsphere, the publisher of NaturalRefrigerants.com, has released “Clean Cooling for Data Centers 2025,” a new report featuring nine articles based on in-depth interviews with cooling system and component manufacturers.
+The report provides an overview of the state of “clean cooling” in the data center sector, defined as mechanical cooling with natural refrigerants, liquid cooling systems that use non-fluorinated refrigerants, heat pumps and the components that make it possible to recover and reuse waste heat, and free cooling via dry, hybrid or evaporative coolers.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45996</v>
+        <v>46048</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>In collaboration with CERN, Swedish-based manufacturer SWEP is supplying brazed plate heat exchangers (BPHE) for the laboratory’s new CO2 (R744)-based cooling system, which includes its Q185H model developed specifically for the project. CERN is updating its ATLAS and CMS sites at the Large Hadron Collider (LHC), located on the France–Switzerland border, in preparation for its fourth operational run, scheduled to begin in 2030. The renovation includes the installation of two new CO2 systems capable of cooling the refrigerant down to −53°C (−63.4°F). To regulate the temperature of the particle detectors in CERN’s new High-Luminosity LHC program, SWEP engineers adapted the company’s B185 BPHE to include a Q-pipe. The newly created Q185H heat exchanger will act as a CO2 evaporator to absorb and remove the increased thermal load resulting from higher radiation levels, according to SWEP. “The entire installation was dimensioned and built specifically to incorporate [our] robust units,” SWEP said. Both its B185 and Q185H BPHEs will “play critical roles” in the cooling system, acting as CO2 superheaters ‒ preventing liquid droplets from entering and damaging compressors ‒ and as CO2 cascades, building a thermal bridge between stages, the company added. The previous refrigeration systems at the ATLAS and CMS sites used synthetic high-GWP-based refrigerants. The new CO2 system is expected to reduce the facility’s greenhouse gas emissions by 40,000 metric tons of CO2e per year, according to CERN. CO2 system details: The combined 1.3MW (370TR) cooling system features 18 modules, seven installed at ATLAS and 11 at CMS, each supplying 70kW (20TR) of capacity.  Due to the lack of space around the detectors, the cooling system, positioned on the surface, will pipe the −53°C CO2 refrigerant 90m (295ft) underground to the heat exchangers. “The unique properties of CO2 enable the use of small pipes ‒ a significant advantage where space is limited,” SWEP said. The cooling systems represent a novel combination of subcritical and transcritical CO2 technologies, said Dirk Leuteritz, Head of Sales at Compact Kältetechnik ‒ the German company that helped develop the solution.  CO2 evaporator: With a vertical tube for rising vapor and a separate tube for descending condensate, the Q185H heat exchanger will maintain the temperature of the detectors below −25°C (−13°F), as required.  The design passively transfers heat, with high temperatures from the radiation detector boiling a two–phase liquid fluid, like helium or nitrogen. The resulting vapor rises through the Q-pipe to the upper end of the BPHE, where the −53°C CO2 refrigerant rejects the heat. Gravity pulls the condensed liquid back into contact with the heat from the detector, restarting the evaporation cycle.  Moving the market: In 2005 SWEP developed its first high-pressure CO2 heat exchanger for CERN’s LHC beauty, or bottom quark, experiment using CO2 cooling.  As a result of the collaboration, SWEP introduced its reinforced B16DW CO2 heat exchanger to the refrigeration market.  Quotable: “We [have] pushed the boundaries of what can be achieved with CO2 natural refrigerant,“ said Yann Herpin, Cooling Engineer at CERN. “We are proud to say that this new system is paving the way for further developments in CO2 refrigeration technology, which will lead to reduced emissions in many other industrial applications.” “We are proud to say that this new system is paving the way for further developments in CO2 refrigeration technology.” Yann Herpin, Cooling Engineer at CERN</t>
+          <t>ATMOsphere, the publisher of NaturalRefrigerants.com, has released “Clean Cooling for Data Centers 2025,” a new report featuring nine articles based on in-depth interviews with cooling system and component manufacturers.
+The report provides an overview of the state of “clean cooling” in the data center sector, defined as mechanical cooling with natural refrigerants, liquid cooling systems that use non-fluorinated refrigerants, heat pumps and the components that make it possible to recover and reuse waste heat, and free cooling via dry, hybrid or evaporative coolers. The report also touches on the economic and regulatory forces reshaping the industry’s approach to cooling.
+The report can be downloaded here.
+“Clean Cooling for Data Centers 2025” takes a qualitative approach to assessing the current state of clean cooling in data centers. Articles based on interviews with cooling system and component manufacturers provide the lay of the land and give an idea of what’s next. The following companies were interviewed for the report: Alfa Laval, BAC, Carel, Fenagy, Jaeggi, Kelvion, Secon, SWEP and Zudek.
+“This report is not just a first for ATMOsphere but a first for the data center sector,” said Michael Hines, the report’s lead author. “This is the first report to focus strictly on clean cooling in data centers, and it provides valuable insights into the state of natural refrigerants in the industry.”
+“This report is not just a first for ATMOsphere but a first for the data center sector.”
+Michael Hines
+Lead Author of “Clean Cooling for Data Centers 2025”
+Article previews
+Below is a short look into each of the nine articles that appear in “Clean Cooling for Data Centers 2025,” which can be downloaded for here.
+Alfa Laval: The Swedish manufacturer’s data center business is booming with growing demand for both its gasketed and brazed plate heat exchangers. The company is developing new brazed plate heat exchangers to meet the needs of larger coolant distribution units (CDUs), according to Anna Blomborg, Head of Data Centers at Alfa Laval. “The forecasts we’re seeing are extraordinary,” Blomborg said.
+BAC: Data centers are big business for BAC, but it’s not just the company’s heat rejection technology that is making a mark on the industry. BAC also offers a single-phase immersion cooling system with an in-tank heat exchanger, which is detailed in a case study on a Houston colocation facility.
+Carel: Carel has worked in the data center industry since the 1970s. Enrico Boscaro, in addition to being the company’s Group Marketing Manager for HVAC Industrial, is also the Chairman of Eurovent’s IT Cooling Task Force. He participated in a Q&amp;A discussing the evolution of data center cooling technologies and regulations in the sector.
+Fenagy: Industrial heating and cooling systems manufacturer Fenagy has big plans for the data center sector. The company is particularly interested in the potential of waste heat recovery and is currently working on a project in Kajaani, Finland, where it’s supplying hydrocarbon heat pumps that cool servers, capture waste heat and then lift it for use in the local district heating network.
+Jaeggi: Jaeggi has supplied its hybrid dry coolers to more than 200 data centers since it first broke into the industry in 1996. While much attention has been on the growth of the data center industry in the United States, Jaeggi shared why it’s also bullish on the Australian market.
+Kelvion: Kelvion has worked with data centers for decades, and in the past 10 years its product portfolio has evolved rapidly alongside the industry. Along with his company’s product portfolio of heat rejection solutions, Timo Kivilaht, the SVP of Global Sales and Solutions, discussed Kelvion’s move from the gray space to the white space and how it seeks to help data center operators balance capital and operating expenditures.
+Secon: Hydrocarbon heat pump and chiller manufacturer Secon has completed more than 30 data center projects and is seeing “increased demand in this area,” according to Joachim Schadt, the company’s Managing Director and Owner. One of its recent projects was in Hamburg for European edge data center operator Penta Infra, whose Head of Engineering spoke about why propane (R290) chillers were chosen for the Hamburg facility.
+SWEP: Global heat exchanger manufacturer SWEP sees an opportunity for its heat exchangers to help data centers turn waste heat into energy. Christer Frennfelt, Business Development Manager at SWEP, shared details about a high-performance computing data center in Sweden where its brazed plate heat exchangers facilitate free cooling and heat recovery.
+Zudek: Ammonia (R717) heat pump and chiller manufacturer Zudek has worked on five data centers across South Africa and Germany. Its recently launched air-cooled chiller, the Windmatik, is being targeted at data centers, but it was a project featuring its Airmatik chiller that the company spoke about for its case study.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/swep-heat-exchangers-integral-part-of-new-co2-based-cooling-system-at-cern/</t>
+          <t>https://naturalrefrigerants.com/news/atmosphere-releases-clean-cooling-for-data-centers-2025-a-new-report-featuring-interviews-with-9-cooling-system-and-component-manufacturers/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ATMO Europe: Carel Outlines CO2 and Propane Commercial Refrigeration Evolution and Trends</t>
+          <t>Cencosud, Nestlé and OXXO Colombia to Present at ATMO LATAM 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Samuele Da Ros, Group Solution Marketing Manager for Food Retail Applications at Carel, outlined the evolution and market adoption trends of CO2 (R744) and propane (R290) refrigeration solutions in commercial applications in a presentation at the ATMOsphere (ATMO) Europe Summit 2025. The event, organized by ATMOSphere, was held November 24–25 in Padova, Italy. ATMOsphere is the publisher of NaturalRefrigerants.com. Carel, an Italy-based manufacturer of refrigeration components and controls, offers its products globally through over 30 subsidiaries and affiliates. “Our history with natural refrigerants started over 20 years ago,” Da Ros said. “Through our work supplying components to OEMs, we’ve contributed to the installation of more than 20,000 centralized CO2 systems, over 10,000 CO2 condensing units and 5,000 semi plug-in cases operating on CO2 or propane.” Points highlighted by Da Ros included compact CO2 condensing units, providing more solutions at lower prices, increased adoption of single–circuit architecture for large propane vertical cases and an increased design focus on CO2 evaporator control. Reduced costs: “In large commercial installations, CO2 is the most used refrigerant in Europe,” Da Ros said, noting that ongoing technological improvements now allow CO2 condensing units to be offered at “achievable prices” even for stores under 800m2 (8,610ft2).  The latest developments in CO2 condensing units include double–stage compression and variable speed compressors, which provide ”flexible capacity to efficiently meet low– and medium-temperature [LT/MT] requirements in one single unit,” Da Ros said. When it comes to centralized CO2 systems, he explained that racks smaller than 40kW (11.4TR) of cooling capacity now contain many of the features reserved in the past for larger units, including heat reclaim, two suction lines to enable booster designs and inverter-driven compressors on both suction lines.  New designs: Da Ros reports that in the past three years, large vertical propane cases have started adopting single–circuit architecture, with variable speed compression.  In 2023 Europe accepted the international safety standard IEC (International Electrotechnical Commission) 60335-2-89, which was updated in 2019, to raise the flammable refrigerant charge in a single circuit to 500g. The new design simplifies the unit, reducing capital, operating and maintenance costs. “There is some reluctance to leave the known for the unknown, but the use of single–circuit propane cases with up to 7kW [2TR] of MT cooling capacity or 3kW [0.85TR] of LT is picking up,” Da Ros said.  Next step: “Our latest frontier involves working to optimize and embrace semi-flooded CO2 evaporators,” Da Ros said.  Running on extremely low superheat brings complexity, according to Da Ros, but it also provides efficiency benefits, with higher evaporating temperatures requiring smaller evaporators. “With the proper algorithms, we can control it,” Da Ros said, making CO2 refrigeration even better.  Quotable: “The common thread in the evolution of these systems is to make them easier to install, use and maintain in real–world conditions,” Da Ros said, adding that in Europe, over 80% of Carel’s business supplying food retail refrigeration products involves natural refrigerant components. “The common thread in the evolution of these systems is to make them easier to install, use and maintain in real–world conditions.” Samuele Da Ros, Group Solution Marketing Manager for Food Retail Applications at Carel</t>
+          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has published a preview of the program for ATMOsphere (ATMO) LATAM 2026, which will feature a keynote from leading South America retailer Cencosud as well as presentations from Nestlé and OXXO Colombia, among other end users.
+Cencosud’s Sustainability Manager will kick off ATMO LATAM 2026, set for March 9–10 in Bogotá, by sharing the company’s vision for sustainability and its progress in adopting natural refrigerants.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45987</v>
+        <v>46062</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Samuele Da Ros, Group Solution Marketing Manager for Food Retail Applications at Carel, outlined the evolution and market adoption trends of CO2 (R744) and propane (R290) refrigeration solutions in commercial applications in a presentation at the ATMOsphere (ATMO) Europe Summit 2025. The event, organized by ATMOSphere, was held November 24–25 in Padova, Italy. ATMOsphere is the publisher of NaturalRefrigerants.com. Carel, an Italy-based manufacturer of refrigeration components and controls, offers its products globally through over 30 subsidiaries and affiliates. “Our history with natural refrigerants started over 20 years ago,” Da Ros said. “Through our work supplying components to OEMs, we’ve contributed to the installation of more than 20,000 centralized CO2 systems, over 10,000 CO2 condensing units and 5,000 semi plug-in cases operating on CO2 or propane.” Points highlighted by Da Ros included compact CO2 condensing units, providing more solutions at lower prices, increased adoption of single–circuit architecture for large propane vertical cases and an increased design focus on CO2 evaporator control. Reduced costs: “In large commercial installations, CO2 is the most used refrigerant in Europe,” Da Ros said, noting that ongoing technological improvements now allow CO2 condensing units to be offered at “achievable prices” even for stores under 800m2 (8,610ft2).  The latest developments in CO2 condensing units include double–stage compression and variable speed compressors, which provide ”flexible capacity to efficiently meet low– and medium-temperature [LT/MT] requirements in one single unit,” Da Ros said. When it comes to centralized CO2 systems, he explained that racks smaller than 40kW (11.4TR) of cooling capacity now contain many of the features reserved in the past for larger units, including heat reclaim, two suction lines to enable booster designs and inverter-driven compressors on both suction lines.  New designs: Da Ros reports that in the past three years, large vertical propane cases have started adopting single–circuit architecture, with variable speed compression.  In 2023 Europe accepted the international safety standard IEC (International Electrotechnical Commission) 60335-2-89, which was updated in 2019, to raise the flammable refrigerant charge in a single circuit to 500g. The new design simplifies the unit, reducing capital, operating and maintenance costs. “There is some reluctance to leave the known for the unknown, but the use of single–circuit propane cases with up to 7kW [2TR] of MT cooling capacity or 3kW [0.85TR] of LT is picking up,” Da Ros said.  Next step: “Our latest frontier involves working to optimize and embrace semi-flooded CO2 evaporators,” Da Ros said.  Running on extremely low superheat brings complexity, according to Da Ros, but it also provides efficiency benefits, with higher evaporating temperatures requiring smaller evaporators. “With the proper algorithms, we can control it,” Da Ros said, making CO2 refrigeration even better.  Quotable: “The common thread in the evolution of these systems is to make them easier to install, use and maintain in real–world conditions,” Da Ros said, adding that in Europe, over 80% of Carel’s business supplying food retail refrigeration products involves natural refrigerant components. “The common thread in the evolution of these systems is to make them easier to install, use and maintain in real–world conditions.” Samuele Da Ros, Group Solution Marketing Manager for Food Retail Applications at Carel</t>
+          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has published a preview of the program for ATMOsphere (ATMO) LATAM 2026, which will feature a keynote from leading South America retailer Cencosud as well as presentations from Nestlé and OXXO Colombia, among other end users.
+Cencosud’s Sustainability Manager will kick off ATMO LATAM 2026, set for March 9–10 in Bogotá, by sharing the company’s vision for sustainability and its progress in adopting natural refrigerants. The company operates more than 1,000 supermarkets and has made the “conversion of refrigerant gases” one of its sustainability priorities. It operates 15 stores that use transcritical CO2 (R744) refrigeration systems, according to its 2024 sustainability report.
+Nestlé and contractor Sistemas de Refrigeración Totales will present a critical load ammonia (R717) chiller with adiabatic condensers. OXXO Colombia, Latin America’s largest convenience store chain, will speak on the same panel about its work with natural refrigerants. 
+End users from the agricultural sector will also take the stage at ATMO LATAM 2026. Avo Pak, a Colombian avocado processor, will speak about its use of CO2 refrigeration systems. The joint presentation will also feature contractor SUTRAK and manufacturer Advansor. 
+Contractors and installers will have their own dedicated panel where they will share their experiences with natural refrigerants and outlook on the sector. Chilean contractor Sofrisur and Costa Rican contractor Dicoma Refrigeración are two of the confirmed presenters.
+Get Your Tickets to ATMO LATAM 2026
+Policy and training
+Day two will feature a policy panel covering standards and regulations impacting natural refrigerants in Latin America. It will feature Edwin M. Dickson, Environmental Consultant at Colombia’s Ministry of Environment and Sustainable Development, and Omarly Acevedo, International Consultant, Montreal Protocol and for UNIDO in Latin America. ATMOsphere will also discuss HFOs and the growing threat of PFAS (per- and polyfluoroalkyl substances) and TFA (trifluoroacetic acid).
+Training will also be a topic of discussion on day two of ATMO LATAM. ACAIRE (The Colombian Association of Air-Conditioning and Refrigeration), will headline the training panel with additional participants announced soon. The session will bring together experts to discuss the current state, opportunities and challenges of professional training in natural refrigerants in Latin America.
+The program is still being finalized and will also include sessions dedicated to global and regional market trends. Tickets for ATMO LATAM 2026 are still available and can be purchased here.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-carel-outlines-co2-and-propane-commercial-refrigeration-evolution-and-trends/</t>
+          <t>https://naturalrefrigerants.com/news/cencosud-nestle-and-oxxo-colombia-to-present-at-atmo-latam-2026/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>‘The Middle East Is Ready to Scale Natural Refrigerants,’ Says Epta Middle East General Manager</t>
+          <t>New Zealand Commissions 865kW CO2 Cold Storage Facility Using 2 SCM Frigo Racks</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Middle East has traditionally been a tough market to crack for natural refrigerant-based HVAC&amp;R equipment due to the region’s high ambient temperatures, shortage of trained technicians and lack of regulations restricting the use of f-gases. Epta established itself in the region over a decade ago, and since then it has installed thousands of propane (R290) self-contained cabinets in grocery stores and helped show CO2 (R744) could work in supermarkets there. While the industry is still in its infancy, Andrea Cavalet, Epta’s Middle East General Manager, told NaturalRefrigerants.com that it’s primed for growth. “The Middle East is ready to scale natural refrigerants, but success depends on proving performance in high ambient conditions, investing in people and aligning on pragmatic policies,” Cavalet said. “Epta is committed on all three fronts.” In an attempt to accelerate this transition, ATMOsphere, publisher of NaturalRefrigerants.com, is hosting ATMO Middle East in Abu Dhabi, the United Arab Emirates, from September 7–8 2026. This is ATMOsphere’s first-ever event in the Middle East, and Epta is the platinum sponsor. To set the stage for ATMO Middle East, Cavalet spoke to NaturalRefrigerants.com about Epta’s work in the region, the challenges natural refrigerants face, the strategies for overcoming them and why it decided to take a leading role in the event. Andrea Cavalet, Epta’s Middle East General Manager. Photo credit: Epta What is the current state of Epta’s operations in the Middle East? Andrea Cavalet: Over the last decade, Epta has built a truly regional leadership presence in the Gulf and surrounding markets. The Group operates from hubs in the United Arab Emirates, in the Kingdom of Saudi Arabia, in India with a direct installation and service organization and through certified partners across all of the other different countries, providing full turn-key projects together with leading retailers. In 2025, Epta further diversified activity beyond the GCC [Gulf Cooperation Council] into Lebanon, Iraq and Egypt. In the last five years alone, Epta has delivered solutions to almost 500 stores across the Middle East, covering supermarkets and hypermarkets. Its natural refrigerant portfolio is represented by thousands of self-contained displays running on R290 and by the Group’s reference project: the Carrefour by MAF supermarket in Masdar Sustainable City in Abu Dhabi, running on CO2 since 2019. Continuing this trajectory, another major hypermarket in the UAE, currently undergoing renovation to adopt CO2 technology, is strategically set to open in Q2 2026. What is the current status of natural refrigerants in the Middle East, and how is Epta helping the region transition to naturals? AC: Momentum is building, and we see growing interest among major retailers, especially in the UAE and Kingdom of Saudi Arabia]. This is driven by energy‑efficiency targets and ESG roadmaps, as evidenced by initiatives such as the UAE Climate Law, UAE vision 2040 and Saudi Vision 2030. This ongoing transition is supported by an ecosystem that is steadily maturing, encompassing technical specifications, service expertise, supply chain readiness and the implementation of the Kigali Amendment. Epta’s role is to quickly enable the transition and prove performance in high‑ambient conditions. In the Gulf climate, FTE/ETE/XTE EPTA patented technology enhancements are essential as they stabilize efficiency and capacity when gas cooler outlet temperatures soar. Epta also actively contributes to regional dialogue, e.g., the recent Eurovent Middle East refrigerant transition position paper, and shares field evidence to inform pragmatic timelines and training needs. The Company also invests in capability building, scaling technician-upskilling programs and formal partnerships. These broaden CO2, R290 and safety competencies in the region. “Epta provides technical input to industry working groups, helping ensure that regulatory and transition pathways are aligned with Middle Eastern realities and support a smooth, sustainable adoption of natural refrigerants in the region.” Andrea Cavalet, Middle East General Manager at Epta What are the biggest challenges natural refrigerants face in the Middle East, and what are the strategies for overcoming them? AC: It’s undoubtedly the high ambient conditions. If systems are not carefully engineered to handle these conditions, their efficiency and performance can be significantly affected. The Group’s answer is the FTE/ETE/XTE EPTA architectures that secure performance at high gas‑cooler outlet temperatures. Epta also addresses the critical need for skills and safety readiness. To ensure competence is scaled safely and quickly, Epta has implemented structured training roadmaps and established partnerships with local vocational institutes. Epta acknowledges that the availability of components and perceived CAPEX premia can slow down project decisions. To mitigate this, Epta localizes production where practical, expands its service network and develops comprehensive TCO [total cost of ownership] and TEWI [total equivalent warming impact] business cases that shift the focus from upfront costs to long-term performance, total cost of ownership and environmental impact. Finally, Epta contributes to policy clarity by providing technical input to industry working groups, helping ensure that regulatory and transition pathways are aligned with Middle Eastern realities and support a smooth, sustainable adoption of natural refrigerants in the region. What is the training landscape like for HVAC&amp;R technicians in the Middle East? AC: It’s evolving and moving from a fragmented approach toward a more structured and consistent framework. While CO2 competence remains variable, initiatives are accelerating.  Epta is developing targeted programs, partnering with institutes to build local capability on installation, commissioning, safety and service for CO2 and hydrocarbons. The Group is investing in dedicated workshops and training centers as part of its strategy to raise after‑sales competencies and to ensure reliable lifecycle support for natural refrigerant systems.  These efforts help create a larger pool of certified technicians, a key factor in enabling the responsible scaling of natural refrigerants. Epta is the platinum sponsor of ATMO Middle East. Why did the company decide to play such a large role in this event? AC: Epta took on a leading role at ATMO Middle East because the event convenes decision‑makers who can accelerate a safe, evidence‑based transition to naturals in the Middle East. This commitment embodies Epta’s purpose, “Preserving our planet with conscious innovation, together.” Epta aims to promote solutions that minimize environmental impact, ensure food quality and foster partnerships across industry, research and retail to advance responsible, forward-looking refrigeration. Internally Epta framed ATMO as an opportunity to engage and influence local policymakers on green solutions while showcasing our latest high‑ambient CO2 innovations and field results. Ultimately, the Group also wants to introduce Epta’s integrated proposition to a Middle East audience, complete systems plus end‑to‑end services, reflecting how the Company presents itself globally.</t>
+          <t>SCM Ref NZ, a division of Beijer Ref, has assisted New Zealand refrigeration contractor Technicool Refrigeration with the commissioning of a 865kW (246TR) CO2 (R744) refrigeration facility owned by Manawatu Cold Storage that features two racks manufactured by fellow group member SCM Frigo.
+The smaller rack supports 135kW (38.4TR) of frozen cold storage capacity at −20°C (−4°F) and 70kW (19.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45999</v>
+        <v>46057</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The Middle East has traditionally been a tough market to crack for natural refrigerant-based HVAC&amp;R equipment due to the region’s high ambient temperatures, shortage of trained technicians and lack of regulations restricting the use of f-gases. Epta established itself in the region over a decade ago, and since then it has installed thousands of propane (R290) self-contained cabinets in grocery stores and helped show CO2 (R744) could work in supermarkets there. While the industry is still in its infancy, Andrea Cavalet, Epta’s Middle East General Manager, told NaturalRefrigerants.com that it’s primed for growth. “The Middle East is ready to scale natural refrigerants, but success depends on proving performance in high ambient conditions, investing in people and aligning on pragmatic policies,” Cavalet said. “Epta is committed on all three fronts.” In an attempt to accelerate this transition, ATMOsphere, publisher of NaturalRefrigerants.com, is hosting ATMO Middle East in Abu Dhabi, the United Arab Emirates, from September 7–8 2026. This is ATMOsphere’s first-ever event in the Middle East, and Epta is the platinum sponsor. To set the stage for ATMO Middle East, Cavalet spoke to NaturalRefrigerants.com about Epta’s work in the region, the challenges natural refrigerants face, the strategies for overcoming them and why it decided to take a leading role in the event. Andrea Cavalet, Epta’s Middle East General Manager. Photo credit: Epta What is the current state of Epta’s operations in the Middle East? Andrea Cavalet: Over the last decade, Epta has built a truly regional leadership presence in the Gulf and surrounding markets. The Group operates from hubs in the United Arab Emirates, in the Kingdom of Saudi Arabia, in India with a direct installation and service organization and through certified partners across all of the other different countries, providing full turn-key projects together with leading retailers. In 2025, Epta further diversified activity beyond the GCC [Gulf Cooperation Council] into Lebanon, Iraq and Egypt. In the last five years alone, Epta has delivered solutions to almost 500 stores across the Middle East, covering supermarkets and hypermarkets. Its natural refrigerant portfolio is represented by thousands of self-contained displays running on R290 and by the Group’s reference project: the Carrefour by MAF supermarket in Masdar Sustainable City in Abu Dhabi, running on CO2 since 2019. Continuing this trajectory, another major hypermarket in the UAE, currently undergoing renovation to adopt CO2 technology, is strategically set to open in Q2 2026. What is the current status of natural refrigerants in the Middle East, and how is Epta helping the region transition to naturals? AC: Momentum is building, and we see growing interest among major retailers, especially in the UAE and Kingdom of Saudi Arabia]. This is driven by energy‑efficiency targets and ESG roadmaps, as evidenced by initiatives such as the UAE Climate Law, UAE vision 2040 and Saudi Vision 2030. This ongoing transition is supported by an ecosystem that is steadily maturing, encompassing technical specifications, service expertise, supply chain readiness and the implementation of the Kigali Amendment. Epta’s role is to quickly enable the transition and prove performance in high‑ambient conditions. In the Gulf climate, FTE/ETE/XTE EPTA patented technology enhancements are essential as they stabilize efficiency and capacity when gas cooler outlet temperatures soar. Epta also actively contributes to regional dialogue, e.g., the recent Eurovent Middle East refrigerant transition position paper, and shares field evidence to inform pragmatic timelines and training needs. The Company also invests in capability building, scaling technician-upskilling programs and formal partnerships. These broaden CO2, R290 and safety competencies in the region. “Epta provides technical input to industry working groups, helping ensure that regulatory and transition pathways are aligned with Middle Eastern realities and support a smooth, sustainable adoption of natural refrigerants in the region.” Andrea Cavalet, Middle East General Manager at Epta What are the biggest challenges natural refrigerants face in the Middle East, and what are the strategies for overcoming them? AC: It’s undoubtedly the high ambient conditions. If systems are not carefully engineered to handle these conditions, their efficiency and performance can be significantly affected. The Group’s answer is the FTE/ETE/XTE EPTA architectures that secure performance at high gas‑cooler outlet temperatures. Epta also addresses the critical need for skills and safety readiness. To ensure competence is scaled safely and quickly, Epta has implemented structured training roadmaps and established partnerships with local vocational institutes. Epta acknowledges that the availability of components and perceived CAPEX premia can slow down project decisions. To mitigate this, Epta localizes production where practical, expands its service network and develops comprehensive TCO [total cost of ownership] and TEWI [total equivalent warming impact] business cases that shift the focus from upfront costs to long-term performance, total cost of ownership and environmental impact. Finally, Epta contributes to policy clarity by providing technical input to industry working groups, helping ensure that regulatory and transition pathways are aligned with Middle Eastern realities and support a smooth, sustainable adoption of natural refrigerants in the region. What is the training landscape like for HVAC&amp;R technicians in the Middle East? AC: It’s evolving and moving from a fragmented approach toward a more structured and consistent framework. While CO2 competence remains variable, initiatives are accelerating.  Epta is developing targeted programs, partnering with institutes to build local capability on installation, commissioning, safety and service for CO2 and hydrocarbons. The Group is investing in dedicated workshops and training centers as part of its strategy to raise after‑sales competencies and to ensure reliable lifecycle support for natural refrigerant systems.  These efforts help create a larger pool of certified technicians, a key factor in enabling the responsible scaling of natural refrigerants. Epta is the platinum sponsor of ATMO Middle East. Why did the company decide to play such a large role in this event? AC: Epta took on a leading role at ATMO Middle East because the event convenes decision‑makers who can accelerate a safe, evidence‑based transition to naturals in the Middle East. This commitment embodies Epta’s purpose, “Preserving our planet with conscious innovation, together.” Epta aims to promote solutions that minimize environmental impact, ensure food quality and foster partnerships across industry, research and retail to advance responsible, forward-looking refrigeration. Internally Epta framed ATMO as an opportunity to engage and influence local policymakers on green solutions while showcasing our latest high‑ambient CO2 innovations and field results. Ultimately, the Group also wants to introduce Epta’s integrated proposition to a Middle East audience, complete systems plus end‑to‑end services, reflecting how the Company presents itself globally.</t>
+          <t>SCM Ref NZ, a division of Beijer Ref, has assisted New Zealand refrigeration contractor Technicool Refrigeration with the commissioning of a 865kW (246TR) CO2 (R744) refrigeration facility owned by Manawatu Cold Storage that features two racks manufactured by fellow group member SCM Frigo.
+The smaller rack supports 135kW (38.4TR) of frozen cold storage capacity at −20°C (−4°F) and 70kW (19.9TR) of capacity at 5°C (41°F) for the environmental loading area, Chris Gibbons, Product Development Manager at SCM Ref NZ, told NaturalRefrigerants.com. The other rack supplies 660kW (187.7TR) of blast freezing capacity at −30°C (−22°F).
+“This project showcases the increased interest and movement of R744 into industrial markets that are predominantly ammonia [R717] and to a lesser extent synthetics in NZ,” Gibbons said. “The end user has already entered discussions regarding CO2 in its next cold store project.”
+Additional details: The 80bar (1,160psi) design pressure rating across all the medium– and low-temperature suction groups enables pressure containment during loss-of-power events, eliminating the requirement for resilience units or generators, according to Gibbons.
+When operating at full refrigeration capacity, the system can recover a maximum of 250kW (71.1TR) of heating capacity from the blast freezer rack and 100kW (28.4TR) from the smaller unit for glycol defrosting and underfloor heating.
+“The blast freezer rack — an impressive installation with 14 compressors — operates remarkably quietly at full capacity, especially compared to equivalent synthetic or ammonia systems,” Gibbons said.
+Expanding market: With daily summer ambient temperatures in New Zealand averaging between 20 and 28°C (68 and 82°F), interest in CO2 continues to grow in the region.
+The project brings SCM Ref NZ’s total number of R744 installations in the country to 82 by the end of 2025, Gibbons said. It includes 37 industrial–sized racks and 45 commercial projects.
+CO2 installations in NZ in the mid-2010s were limited to supermarkets. Today its use spans a wide range of sectors from small stores to industrial applications.
+New product: In 2025 SCM Ref NZ built a CO2 ice builder for use in the country’s expansive dairy industry.
+SCM Ref NZ designed and constructed the evaporator coils using K65 copper piping and linked the unit to its New Zealand-built SMTDX10 transcritical CO2 refrigeration pack.
+The unit takes advantage of off-peak energy rates by generating and storing up to 500kg (1,100lbs) of ice.
+Quotable: “Following the success of our 2022 series run, we are organizing another NZ-wide CO2 roadshow with stops at nine venues to introduce transcritical CO2 as a safe natural future-proof refrigerant,” Gibbons said. “ With live plant demonstrations, it’s a chance for engineers and end users to discover the advantages of R744, how it works and what is currently available. With the increasing interest, I am confident it will create more R744 opportunities.”
+“The end user has already entered discussions regarding CO2 in its next cold store project.”
+Chris Gibbons, Product Development Manager at SCM Ref NZ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/the-middle-east-is-ready-to-scale-natural-refrigerants-says-epta-middle-east-general-manager/</t>
+          <t>https://naturalrefrigerants.com/news/new-zealand-commissions-865kw-co2-cold-storage-facility-using-2-scm-frigo-racks/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ATMO America 2026 Is Set for June 2–3 in New York City</t>
+          <t>Scantec Supplies 1.13MW Low-Charge DX Ammonia System for New Melbourne Cold Storage Facility</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has announced that the 15th edition of the ATMOsphere (ATMO) America Summit 2026 will be held in New York City June 2–3 and registration is open. This is the first time ATMO America will be held in New York City. Last year’s ATMO America conference was held in Atlanta. “We wanted to make it easy for all end users, regulators, contractors and manufacturers to attend and engage over two exciting days of conference and business matchmaking,” said Marc Chasserot, CEO and Founder of ATMOsphere. This 15th annual edition of ATMO America will gather key industry experts, including manufacturers, policymakers, end users and contractors, to learn about the latest developments in natural refrigerant-based HVAC&amp;R systems, including those using CO2 (R744), hydrocarbons and ammonia (R717). The program for ATMO America 2026 is still being assembled and registration will open soon. The program from ATMO America 2025 can be found here. Want to stay updated about ATMO America 2026? Subscribe to ATMOsphere’s events newsletter You can now register for the event here and find the preliminary program and other information on the event website. ATMOsphere is offering a holiday discount of up to $250 (€214) on standard tickets until January 4. End users can register for free, as can government personnel, employees of non-governmental organizations (NGOs) and members of the press. Contractors/installers of HVAC&amp;R systems are eligible to receive one free ticket per organization, with a 50% discount on additional tickets. The Platinum sponsor of ATMO America 2026 is Hillphoenix. Gold sponsors are Copeland, Hussmann and Kysor Warren Epta US. Additional sponsorship opportunities are available, and those interested in sponsoring the event can find more information here and by contacting ATMOsphere’s Partnership Manager Silvia Scaldaferri at silvia.scaldaferri@shecco.com.</t>
+          <t>Australian Scantec Refrigeration Technologies has supplied a 1.13MW (321TR) low-charge DX ammonia (R717) system for a new Melbourne cold storage facility, featuring Grasso V1800 10-cylinder reciprocating compressors manufactured by GEA Heating &amp; Refrigeration Technologies.
+The system supplies cooling for a 2°C (36°F) temperature staging area and four dual-duty rooms, each capable of operating as either a chiller at 0°C (32°F) or a freezer at −25°C (−13°F), Stefan Jensen, Scantec’s Managing Director, told NaturalRefrigerants.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46001</v>
+        <v>46050</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has announced that the 15th edition of the ATMOsphere (ATMO) America Summit 2026 will be held in New York City June 2–3 and registration is open. This is the first time ATMO America will be held in New York City. Last year’s ATMO America conference was held in Atlanta. “We wanted to make it easy for all end users, regulators, contractors and manufacturers to attend and engage over two exciting days of conference and business matchmaking,” said Marc Chasserot, CEO and Founder of ATMOsphere. This 15th annual edition of ATMO America will gather key industry experts, including manufacturers, policymakers, end users and contractors, to learn about the latest developments in natural refrigerant-based HVAC&amp;R systems, including those using CO2 (R744), hydrocarbons and ammonia (R717). The program for ATMO America 2026 is still being assembled and registration will open soon. The program from ATMO America 2025 can be found here. Want to stay updated about ATMO America 2026? Subscribe to ATMOsphere’s events newsletter You can now register for the event here and find the preliminary program and other information on the event website. ATMOsphere is offering a holiday discount of up to $250 (€214) on standard tickets until January 4. End users can register for free, as can government personnel, employees of non-governmental organizations (NGOs) and members of the press. Contractors/installers of HVAC&amp;R systems are eligible to receive one free ticket per organization, with a 50% discount on additional tickets. The Platinum sponsor of ATMO America 2026 is Hillphoenix. Gold sponsors are Copeland, Hussmann and Kysor Warren Epta US. Additional sponsorship opportunities are available, and those interested in sponsoring the event can find more information here and by contacting ATMOsphere’s Partnership Manager Silvia Scaldaferri at silvia.scaldaferri@shecco.com.</t>
+          <t>Australian Scantec Refrigeration Technologies has supplied a 1.13MW (321TR) low-charge DX ammonia (R717) system for a new Melbourne cold storage facility, featuring Grasso V1800 10-cylinder reciprocating compressors manufactured by GEA Heating &amp; Refrigeration Technologies.
+The system supplies cooling for a 2°C (36°F) temperature staging area and four dual-duty rooms, each capable of operating as either a chiller at 0°C (32°F) or a freezer at −25°C (−13°F), Stefan Jensen, Scantec’s Managing Director, told NaturalRefrigerants.com. When all four dual-duty rooms operate as freezers, the total refrigeration load is 742 kW (211TR) for the chambers, with the staging area supplying an additional 384 kW (109TR) of cooling capacity.
+“Using ammonia in a centralized, low–charge refrigerating plant is an environmental contribution second to none, delivering PFAS–free, zero ODP, and zero GWP refrigeration performance with a predicted SEC of only 8‒9kWh per cubic meter per year,” said Greg Clements, GEA’s Sales Manager for Australia and the APAC region.
+Additional details: Scantec designed, installed and commissioned the ammonia system in the cold warehouse located roughly 10km (8mi) from Melbourne’s city center.
+Together the facility’s 200m (656ft)–long staging area and four dual-duty rooms, with a total area of 22,141m2 (238,323 ft2), deliver 230,000m3 (8,122,400ft3) of cold-storage capacity.
+The design includes heat recovery for underfloor heating, Scantec said.
+The site can experience ambient temperatures that swing over 40°C (104°F) between seasons, according to GEA.
+Optimized design: “Built on 20 years of experience in DX systems, we are confident that this system will be our most energy-efficient yet,” Scantec said, noting that it contains no unnecessary pumps, excessive liquid or receivers.
+“The V1800 delivers excellent part-load performance and a wide variable frequency drive (VFD) range for outstanding energy efficiency with minimal oil carry over, ensuring premium evaporator performance,” Clements said.
+The design cuts annual energy use by over 50% compared with a conventional cold warehouse with an average SEC of 20‒40kWh per cubic meter per year, according to GEA.
+New product: In December 2025 GEA launched a high-pressure screw compressor, Grasso L XHP, optimized for ammonia heat pumps, featuring a design pressure of up to 70bar (1,016psi).
+The new series, available in three models, offers heating capacities from 2 to 11MW (569 to 3,128TR) with a maximum discharge temperature of 140°C (284°F).
+The compressor was installed in early 2024 in a 24MW (6,824TR)-capacity district heating facility at an Estonian combined heat and power plant, according to Kenneth Hoffman, Product Manager at GEA.
+In 2,500 hours of operation, the heat pumps delivered hot water at 47–85°C (116–185°F) to the district heating network with a COP greater than 4, Hoffman reported in a presentation at the ATMOsphere (ATMO) Europe Summit 2024. The event was organized by ATMOsphere, publisher of NaturalRefrigerants.com, and held in Prague, Czech Republic, from November 25–26.
+Quotable: “Capital and operational costs have been reduced thanks to optimized infrastructure and extended service intervals, based on real–time compressor monitoring,” Clements said. “With the compressor system responsible for up to 80% of the total plant power consumption, these improvements contribute to a lower total cost of ownership whilst maintaining high levels of efficiency and reliability.”
+“The V1800 delivers excellent part-load performance and a wide variable frequency drive (VFD) range for outstanding energy efficiency with minimal oil carry over.” 
+Greg Clements, GEA’s Sales Manager for Australia and APAC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-america-2026-is-set-for-june-2-3-in-new-york-city/</t>
+          <t>https://naturalrefrigerants.com/news/scantec-supplies-1-13mw-low-charge-dx-ammonia-system-for-new-melbourne-cold-storage-facility/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ATMO LATAM 2026 Is Set for March 9–10 in Bogotá</t>
+          <t>Natural Refrigerant Chillers Part of Lidl GB’s £43 Million Investment in Retrofits of Over 70 Stores</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has announced that ATMOsphere (ATMO) LATAM 2026 will be held in Bogotá, Colombia, March 9–10. ATMO LATAM 2026 will gather key industry experts, including manufacturers, policymakers, end users and contractors, to learn about the latest developments in natural refrigerant-based HVAC&amp;R systems, including those using CO2 (R744), hydrocarbons and ammonia (R717). The event will also touch on policy developments in the industry and region as well as the latest research on PFAS (per- and polyfluoroalkyl substances).  The tentative program for ATMO LATAM 2026 can be seen here, and registration will open soon. Manufacturers and end users are invited to submit case studies to present at the event. Click here to download the abstract submission template and for the guidelines. Abstracts are due by January 14. ATMO LATAM 2025 was held in Mexico City, and the program from the event can be found here. Want to stay updated about ATMO America 2026? Subscribe to ATMOsphere’s events newsletter Latin America is an emerging market for natural refrigerants. ATMOsphere’s Natural Refrigerants: State of the Industry 2024 report estimated that there were 580 grocery stores and supermarkets in Latin America – defined as Mexico, Central and South America – using transcritical CO2 refrigeration systems. The report also estimated that there were 8.5 million self-contained hydrocarbon (mostly R290) cases installed in food stores in Latin America. Of those 580 transcritical CO2 stores, 80 were in Colombia, with Weston installing the country’s first commercial transcritical CO2 refrigeration system in 2017. In October 2025, Colombian hypermarket chain Alkosto opened its first transcritical CO2 store in Bogotá. The gold sponsor for the event is Hussmann, and the silver sponsors are Güntner and Ice Square. The bronze sponsors are Advansor, Bitzer, Dorin, FB Industrial, GTS, Intarcon, Modine, Sistemas de Refrigeración Totales (SRT), Teklab and Temprite. Those interested in sponsoring the event can find more information here or by contacting ATMOsphere’s Partnership Manager Silvia Scaldaferri at silvia.scaldaferri@shecco.com.</t>
+          <t>Discount retailer Lidl GB, the Great Britain subsidiary of Lidl Germany, has announced plans to modernize over 70 existing stores, with natural refrigerant chillers included in the £43 million ($58 million/€49 million) retrofit investment.
+“The changes to these stores will include new tills and larger freezers to offer a greater range of products,” Lidl said. “[We are] also introducing energy-saving features as part of the modernizations, including chillers that use natural refrigerants and smart lighting systems, to help lower the environmental impact and support Lidl GB’s journey toward net zero.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46002</v>
+        <v>46049</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ATMOsphere, publisher of NaturalRefrigerants.com, has announced that ATMOsphere (ATMO) LATAM 2026 will be held in Bogotá, Colombia, March 9–10. ATMO LATAM 2026 will gather key industry experts, including manufacturers, policymakers, end users and contractors, to learn about the latest developments in natural refrigerant-based HVAC&amp;R systems, including those using CO2 (R744), hydrocarbons and ammonia (R717). The event will also touch on policy developments in the industry and region as well as the latest research on PFAS (per- and polyfluoroalkyl substances).  The tentative program for ATMO LATAM 2026 can be seen here, and registration will open soon. Manufacturers and end users are invited to submit case studies to present at the event. Click here to download the abstract submission template and for the guidelines. Abstracts are due by January 14. ATMO LATAM 2025 was held in Mexico City, and the program from the event can be found here. Want to stay updated about ATMO America 2026? Subscribe to ATMOsphere’s events newsletter Latin America is an emerging market for natural refrigerants. ATMOsphere’s Natural Refrigerants: State of the Industry 2024 report estimated that there were 580 grocery stores and supermarkets in Latin America – defined as Mexico, Central and South America – using transcritical CO2 refrigeration systems. The report also estimated that there were 8.5 million self-contained hydrocarbon (mostly R290) cases installed in food stores in Latin America. Of those 580 transcritical CO2 stores, 80 were in Colombia, with Weston installing the country’s first commercial transcritical CO2 refrigeration system in 2017. In October 2025, Colombian hypermarket chain Alkosto opened its first transcritical CO2 store in Bogotá. The gold sponsor for the event is Hussmann, and the silver sponsors are Güntner and Ice Square. The bronze sponsors are Advansor, Bitzer, Dorin, FB Industrial, GTS, Intarcon, Modine, Sistemas de Refrigeración Totales (SRT), Teklab and Temprite. Those interested in sponsoring the event can find more information here or by contacting ATMOsphere’s Partnership Manager Silvia Scaldaferri at silvia.scaldaferri@shecco.com.</t>
+          <t>Discount retailer Lidl GB, the Great Britain subsidiary of Lidl Germany, has announced plans to modernize over 70 existing stores, with natural refrigerant chillers included in the £43 million ($58 million/€49 million) retrofit investment.
+“The changes to these stores will include new tills and larger freezers to offer a greater range of products,” Lidl said. “[We are] also introducing energy-saving features as part of the modernizations, including chillers that use natural refrigerants and smart lighting systems, to help lower the environmental impact and support Lidl GB’s journey toward net zero.”
+The retailer opened its first store in the U.K. in 1994. Lidl GB marked its 1,000th store milestone on November 27, 2025, with the opening of its East Grinstead, West Sussex, location. In early 2026, the Great Britain subsidiary plans to open 19 new stores.
+Early adopters: To lower its greenhouse gas emissions, Lidl GB noted in its 2017/2018 sustainability report that it was rolling out the use of natural refrigerants across its portfolio, with refrigeration accounting for half of its energy consumption.
+At that time, Lidl GB reported that 50% of its newly installed retail floor refrigeration equipment and 100% of its new and refurbished warehouse refrigeration systems used natural refrigerants.
+In 2018, 83 stores used a bespoke low-energy refrigeration compressor pack combined with an air-source heat pump. The configuration reduced total store energy consumption by 27% compared to the company’s previous operations.
+In 2016, Lidl Germany committed to using propane (R290) plug-in refrigerated units in all future stores across Europe. At Chillventa 2022, Markus Lenz, Director of Marketing and Refrigeration and Integrated Products at Emerson indicated that Lidl also specifies CO2 (R744) refrigeration.
+Sustainability goals: By 2030, Lidl GB aims to reduce its Scope 1 and Scope 2 CO2e emissions by 70% from its 2019 baseline as part of its parent company’s overall 2050 net-zero target.
+Major contributors to the company’s Scope 1 emissions include refrigerant GWP and refrigerant leaks. Lidl GB’s 2021/2022 sustainability report indicates that refrigerant leaks accounted for 10,273 metric tons of CO2e emissions in 2019. By 2022 it had reduced refrigerant emissions by 42%, curtailing them to 5,943 metric tons of CO2e.
+Its total Scope 1 emissions dropped 30% from its 2019 baseline of 22,170 metric tons of CO2e to 15,539 metric tons in 2022.
+Quotable: “We’re starting the new year as we mean to go on, with a major investment that reinforces our commitment to delivering the best experience for customers and creating a positive impact for the communities we serve,” said Lidl GB’s Chief Real Estate Officer Richard Taylor.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-latam-2026-is-set-for-march-9-10-in-bogota/</t>
+          <t>https://naturalrefrigerants.com/news/natural-refrigerant-chillers-part-of-lidl-gbs-43-million-investment-in-retrofits-of-over-70-stores/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ATMO Europe: Danfoss Details How Hydrocarbon High-Temperature Heat Pumps Are Decarbonizing the Food and Beverage Industry</t>
+          <t>Numerous CO2-Based Products to be Featured at AHR Expo 2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hydrocarbon high-temperature heat pumps (HTHP) with outlet temperatures up to 120°C (248°F) are already decarbonizing the food and beverage industry, according to Danfoss. Ivan Rangelov, Industrial Heat Pump Manager at Danfoss, shared details about the technology readiness levels of various HTHPs at the ATMOsphere (ATMO) Europe Summit 2025. ATMOsphere, the publisher of NaturalRefrigerants.com, hosted the event, which was held November 24–25 in Padua, Italy. Wil van den Kerkhof, Technical Director of Dutch OEM Servex, joined Rangelov to present a 1.5MW (427TR) integrated hydrocarbon system for a brewery, delivering steam at up to 130°C (266°F). “With its need for refrigeration and processing temperatures up to 150°C [302°F], the food and beverage industry represents the lowest-hanging fruit for decarbonizing with HTHPs,” Rangelov said. Market-ready units: Danfoss has already launched industrial hydrocarbon compressors using scroll, semi-hermetic piston and screw technologies.  The isobutane (R600a) scroll PSG range provides water temperatures up to 100°C (212°F) with heating capacities ranging from 80 to 500kW (22.7 to 142TR). Its HG66 BOCK R600a semi-hermetic piston compressor provides water temperatures up to 120°C, with heating capacities from 100kW to 1MW (28.4 to 284TR). “Next year we will launch this compressor with butane to produce temperatures up to 135°C [275°F],” Rangelov said. For larger heating capacities from 250kW to 1.5MW (71 to 427TR), Danfoss offers its new KS screw compressor range with integrated inverter technology, using R600a or R290 (propane) refrigerant, with outlet temperatures of up to 100°C.  Case study: Servex designed a 1.5MW hydrocarbon refrigeration/heating system for Gulpener, a brewery in the Netherlands, using Danfoss hydrocarbon compressors. The brewery aims to operate fossil free by 2030.
-  The system includes a 500kW R290 chiller for refrigeration, a second-stage 500kW R600a heat pump supplying 90°C (194°F) water for industry processes and a third-stage 500kW R600 heat pump generating steam at 130°C. “The clean steam, generated at 1bar [14.5psi] of pressure, is injected directly into the brewer’s processes,” Van den Kerkhof said. When the cooling demand is too low to support the HTHPs, the system uses the air cooler as a heat source, he added.  Under development: “Two months ago we kicked off a project at the Danish Technological Institute [DTI] to build a modular design 500kW hydrocarbon heat pump, capable of delivering steam up to 200°C [392°F],” Rangelov said. The heat pump includes a propane unit producing outlet temperatures up to 50°C (122°F), a butane unit generating between 130 and 140°C (266 to 284°F) steam and an MVR (mechanical vapor recompression) cycle to reach 200°C.  With a target to develop a 1MW capacity heat pump, the three-year Danish government EUDP (Energy Technology Development and Demonstration Program) funded project will test a Danfoss piston and a screw compressor in the same application. Danish manufacturer Fenagy will build the unit, and DTI will test it, according to Rangelov. He added that the unit will eventually be installed in a pharmaceutical manufacturing facility owned by the biotechnical firm Fujifilm. “Between the two different compressor types, DTI will determine which technology better fits given applications based on the matrix of COPs,” Rangelov said.  Quotable: “We see a big demand for hydrocarbon heat pumps to address temperatures above 100°C,” Rangelov said. “It’s a good natural choice with the ability to produce temperatures of 130–140°C when condensing at 28bar [406psi].</t>
+          <t>A wide range of equipment designed for CO2 (R744) – including heat pumps, racks, a condensing unit, compressors, valves, tubes and oil separators – will be showcased at the AHR Expo (International Air-Conditioning, Heating, Refrigerating Exposition), scheduled for February 2–4, 2026, in Las Vegas, Nevada.
+The AHR Expo is co-sponsored by ASHRAE and AHRI and is held concurrently with ASHRAE’s Winter Conference. Last year in Orlando, Florida, it attracted 50,807 attendees and 1,878 exhibitors.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45994</v>
+        <v>46045</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hydrocarbon high-temperature heat pumps (HTHP) with outlet temperatures up to 120°C (248°F) are already decarbonizing the food and beverage industry, according to Danfoss. Ivan Rangelov, Industrial Heat Pump Manager at Danfoss, shared details about the technology readiness levels of various HTHPs at the ATMOsphere (ATMO) Europe Summit 2025. ATMOsphere, the publisher of NaturalRefrigerants.com, hosted the event, which was held November 24–25 in Padua, Italy. Wil van den Kerkhof, Technical Director of Dutch OEM Servex, joined Rangelov to present a 1.5MW (427TR) integrated hydrocarbon system for a brewery, delivering steam at up to 130°C (266°F). “With its need for refrigeration and processing temperatures up to 150°C [302°F], the food and beverage industry represents the lowest-hanging fruit for decarbonizing with HTHPs,” Rangelov said. Market-ready units: Danfoss has already launched industrial hydrocarbon compressors using scroll, semi-hermetic piston and screw technologies.  The isobutane (R600a) scroll PSG range provides water temperatures up to 100°C (212°F) with heating capacities ranging from 80 to 500kW (22.7 to 142TR). Its HG66 BOCK R600a semi-hermetic piston compressor provides water temperatures up to 120°C, with heating capacities from 100kW to 1MW (28.4 to 284TR). “Next year we will launch this compressor with butane to produce temperatures up to 135°C [275°F],” Rangelov said. For larger heating capacities from 250kW to 1.5MW (71 to 427TR), Danfoss offers its new KS screw compressor range with integrated inverter technology, using R600a or R290 (propane) refrigerant, with outlet temperatures of up to 100°C.  Case study: Servex designed a 1.5MW hydrocarbon refrigeration/heating system for Gulpener, a brewery in the Netherlands, using Danfoss hydrocarbon compressors. The brewery aims to operate fossil free by 2030.
-  The system includes a 500kW R290 chiller for refrigeration, a second-stage 500kW R600a heat pump supplying 90°C (194°F) water for industry processes and a third-stage 500kW R600 heat pump generating steam at 130°C. “The clean steam, generated at 1bar [14.5psi] of pressure, is injected directly into the brewer’s processes,” Van den Kerkhof said. When the cooling demand is too low to support the HTHPs, the system uses the air cooler as a heat source, he added.  Under development: “Two months ago we kicked off a project at the Danish Technological Institute [DTI] to build a modular design 500kW hydrocarbon heat pump, capable of delivering steam up to 200°C [392°F],” Rangelov said. The heat pump includes a propane unit producing outlet temperatures up to 50°C (122°F), a butane unit generating between 130 and 140°C (266 to 284°F) steam and an MVR (mechanical vapor recompression) cycle to reach 200°C.  With a target to develop a 1MW capacity heat pump, the three-year Danish government EUDP (Energy Technology Development and Demonstration Program) funded project will test a Danfoss piston and a screw compressor in the same application. Danish manufacturer Fenagy will build the unit, and DTI will test it, according to Rangelov. He added that the unit will eventually be installed in a pharmaceutical manufacturing facility owned by the biotechnical firm Fujifilm. “Between the two different compressor types, DTI will determine which technology better fits given applications based on the matrix of COPs,” Rangelov said.  Quotable: “We see a big demand for hydrocarbon heat pumps to address temperatures above 100°C,” Rangelov said. “It’s a good natural choice with the ability to produce temperatures of 130–140°C when condensing at 28bar [406psi].</t>
+          <t>A wide range of equipment designed for CO2 (R744) – including heat pumps, racks, a condensing unit, compressors, valves, tubes and oil separators – will be showcased at the AHR Expo (International Air-Conditioning, Heating, Refrigerating Exposition), scheduled for February 2–4, 2026, in Las Vegas, Nevada.
+The AHR Expo is co-sponsored by ASHRAE and AHRI and is held concurrently with ASHRAE’s Winter Conference. Last year in Orlando, Florida, it attracted 50,807 attendees and 1,878 exhibitors.
+The following are examples of exhibitors with products designed for natural refrigerants, primarily CO2 but also ammonia (R717) and hydrocarbons like propane (R290).
+NDL Industries (booth C2104)
+NDL Industries will exhibit a suite of products for CO2 refrigeration systems, including copper fittings, ball valves, check valves and NDL’s new three-way valves. NDL’s CO2 ball valves and check valves are designed to withstand pressures up to 140bar [2,030psi]. NDL will also highlight its DN65 stainless steel CO2 ball valve, which is capable of handling pressures up to 130bar [1,885psi] and notable for its substantial size and suitability for large-scale CO2 applications.
+In addition, NDL will feature its CO2 copper fittings rated up to 130bar as well as CO2 service tees designed specifically for installing service valves with 10mm [3/8in] stainless steel stubs.
+Danfoss (booth C4907)
+Danfoss will feature its Optyma iCO2 condensing unit, a high-performance outdoor condensing unit engineered for low- or medium-temperature transcritical refrigeration and air-conditioning applications. It is designed for distributed architectures in new supermarkets, equipment upgrades, store expansions/remodels and new refrigerated merchandising programs. Engineered to operate efficiently in ambient temperatures up to 43°C (109°F), the condensing unit combines a hermetic, inverter-driven compressor with scroll and rotary mechanisms, and it comes with service valves, a liquid bypass valve and an oil separator.
+Danfoss also offers the BOCK HGX56 CO2 T, a 6-cylinder transcritical CO2 compressor, winner of the AHR Expo’s 2025 Innovation Award in the refrigeration category. The HGX56 CO2 T is a semi-hermetic compressor designed for industrial refrigeration, cold storage, ice sports facilities and heat pumps, including process and district heating applications.
+Copeland (booth C3607)
+Copeland was named the winner of the 2026 AHR Expo Innovation Award in the refrigeration category for its transcritical CO2 scroll compressors with dynamic vapor injection (DVI) technology. Copeland’s transcritical CO2 scroll compressors are designed for medium-temperature, distributed CO2 refrigeration in small supermarkets and convenience stores. They feature dynamic vapor injection technology, which enhances efficiency and simplifies design, said the announcement. Copeland also offers low-temperature subcritical CO2 scroll compressors.
+ For example, the ZTI scroll compressor is designed for use in transcritical CO2 medium-temperature refrigeration systems, with a standstill pressure of 110bar (1,595psi) and capacities from 7.7 to 18.6kW (2.2 to 5.3TR).
+Castel ( booth SL2415)
+Castel offers a wide range of components for CO2 systems – what it calls the GO GREEN line – including  expansion valves, solenoid valves, safety devices, check valves, pressure regulators, oil control systems and vibration absorbers.
+The products are specifically designed, tested and manufactured for CO2 refrigeration systems, accounting for the high operating pressures and typical working conditions of R744 applications.
+Temprite (booth SU1050)
+Temprite offers coalescent and conventional oil separators, oil reservoirs, drier housings, liquid receivers, suction accumulators and other refrigerant and oil management products for refrigeration and heat pump systems that use ammonia, CO2 and hydrocarbons. Temprite’s oil separators can be used in ultra-low-temperature freezers.
+Westermeyer (booth C4019)
+Westermeyer’s TOS-series CO2 centrifugal oil separator is designed to operate at transcritical pressures in CO2 refrigeration systems. Centrifugal oil separators can remove large quantities of oil from refrigerant at a wide range of operating capacities.
+Noritz America (booth C4929)
+Noritz Corporation and the Nihon Itomic Co., Ltd will showcase their new jointly developed CO2 heat pump water heater for the North American market. Nihon Itomic will lead product development while RB Corporation, a company in the Noritz Group, will handle manufacturing. Noritz America will oversee sales and distribution.
+Vitalis (booth SU369)
+Vitalis will feature its Roxsta CO2 refrigeration system with single-rack capacities up to 960kW (273TR), leveraging technology from German sister company Teko. Equipped with transcritical and subcritical compressors, it is designed for discount stores, supermarkets, commercial kitchens, refrigerated warehouses and industrial processes. Optional heat recovery is included. Vitalis also makes R744 chillers and heat pumps for commercial, industrial, and district energy applications.
+Dorin (booth SL932)
+Dorin USA was a finalist in the refrigeration category of the 2026 AHR Expo Innovation Award competition for its CD700 Range of CO2 transcritical compressors. The 8-cylinder compressors feature motors up to 220 HP  and displacement up to 100m3/h (3,531ft3/h), making it possible to “significantly decrease racks amounts for a given duty, keeping machinery rooms smaller and sensibly decreasing CAPEX,” Dorin said. The CD700 line also features an external discharge manifold, facilitating longer compressor lifetimes, higher efficiency and lower oil temperatures, the company added.
+Baltimore Aircoil (C4507)
+Baltimore Aircoil (BAC) will showcase its Nexus modular hybrid cooler with PuriStream water treatment system for HVAC and light industrial applications; with hybrid, evaporative, and dry capability it employs touchscreen controls that balance water and energy use.
+BAC will also feature a data center-focused model that integrates indoor immersion technology with its broad portfolio of outdoor evaporative, hybrid, adiabatic and dry systems; together, these solutions form the COBALT immersion cooling system. The company was recognized as a 2026 AHR Expo Innovation Award finalist in the cooling category for its upgraded immersion cooling tank, powered by CorTex technology using dielectric fluid.
+SWEP (booth C7121)
+SWEP, part of the Dover Corporation, features brazed plate heat exchangers for HVAC and industrial applications. Most SWEP heat exchangers are available as either copper-brazed or 100% stainless steel single- and multi-pass units. Plate packages can be customized to supply specific thermal characteristics.
+Wieland (booth SU844)
+Wieland offers copper and copper-alloy finned tubes that serve as components in heat exchangers. Tube surfaces are optimized to specific heat transfer requirements.
+Sanhua (booth C900)
+Sanhua offers a wide range of components for commercial refrigeration, including thermostatic and electronic expansion valves, solenoid valves, controllers, pressure sensors and heat exchangers. Its product range is optimized for natural refrigerants such as R290 and CO₂. Sanhua’s brazed plate heat exchangers are suitable for flammable refrigerants, and its heat exchangers can be used in heat pumps, chillers and heating circuits.
+Intellihot (booth SL1620)
+Intellihot offers a CO2 tankless heat pump water heater, which it has installed at public schools in Washington, D.C. Intellihot was named a finalist in the heating category in AHR Expo’s 2024 Innovation Awards competition for its new heat pumps.
+ECO2 Systems (SU1013)
+ECO2 Systems is a provider of CO2 heat pump water heaters for the commercial and residential markets in North America. The systems have a COP of over 5.0 and will produce 145/150°F (63/66°C) hot water at all ambient temperatures down to -25°F (-32°C), said the company.
+Podak (SU2332)
+Podak makes CO2 heat pumps that can be used for hot-water production and space heating in factories, restaurants, sports centers, food kitchens, hospitals and residential buildings.  Water temperature can be heated to 98C and COP reaches a peak value of about five When the ambient temperature approaches 30°C, the company said.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-danfoss-details-how-hydrocarbon-high-temperature-heat-pumps-are-decarbonizing-the-food-and-beverage-industry/</t>
+          <t>https://naturalrefrigerants.com/news/numeroous-co2-based-products-to-be-featured-at-ahr-expo-2026/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ATMO Europe: Jaeggi’s Hybrid Dry Coolers to Provide Cooling for 12MW CERN Data Center in Geneva</t>
+          <t>AHR 2026: NDL Industries Details the CO2 Components It’ll be Exhibiting</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hybrid dry coolers, manufactured by Swiss-based Jaeggi Hybridtechnologie (a subsidiary of Güntner), will provide all of the cooling for a CERN (European Organization for Nuclear Research) data center in Geneva, Switzerland, with an installed IT power capacity of 12MW. Ivan Hemmeler, Jaeggi’s Business Development Manager for Spain and Portugal, outlined the mechanical cooling-free system and its power usage effectiveness (PUE) in a presentation at the ATMOsphere (ATMO) Europe Summit 2025. ATMOsphere, publisher of NaturalRefrigerants.com, hosted the event, which was held November 24–25 in Padua, Italy.  PUE measures a data center’s energy efficiency by comparing the facility’s total power usage to that of the information technology equipment, including servers, storage and networks. A PUE of 1 represents theoretical perfection, with no power used for cooling and infrastructure. “By eliminating the chiller, we have removed the most energy-intensive component in traditional data center cooling,” Hemmeler said, with the hybrid dry cooler system providing a PUE of equal to or less than 1.15. “In addition, the technology uses 70% less water than conventional cooling towers, with just 0.379L [0.1gal] per kWh.” The design: A water-glycol loop transports the data center’s IT heat load directly to the hybrid dry coolers, where “massive double stacked” heat exchangers reject it using ambient air for the majority of the year in Geneva’s temperate climate. “The design is so simple, it becomes naturally resilient,” Hemmeler said.  In the event that temperatures rise to 40°C (104°F) during peak summer conditions, the heat exchanger coils are wetted, with the water fully recirculated. “A cascade design saves water while boosting cooling power, with smart controls optimizing operation based on climate and demand,” Hemmeler explained. Although the total system will be 12MW, currently just 8MW are installed. Of that, up to 4MW (1,137TR) of waste heat can be recovered and supplied to nearby CERN buildings for space heating. CERN, Jaeggi and Austrian refrigeration contractor Equans collaborated on the project.  What’s next: “With the units now installed, the real learning starts as we assess system behavior and refine its operation,” Hemmeler said.  Removing glycol is the next step to simplify the design, Hemmeler explained, adding that doing so could increase efficiency by 10‒20%. “We’ve successfully operated glycol-free data centers with Jaeggi [equipment] for 15 years,” he said. Recovering more waste heat from the system would also improve CERN’s PUE, he noted.  CERN and sustainability: CERN won the ATMO Europe 2025 Best-in-Sector/Industrial End User award for its use of a CO2 (R744)-based refrigeration system to cool its new high-luminosity Large Hadron Collider (LHC) program, scheduled to start operating in 2030.  CERN expects its new CO2 cooling system ‒ providing a combined capacity of 1.3MW (370TR) at its ATLAS and CMS particle detectors ‒ to reduce its greenhouse gas emissions by 40,000 metric tons of CO2e per year compared to synthetic alternatives. Swedish-based manufacturer SWEP developed Q185H, a new CO2 brazed plate heat exchanger, for CERN’s high-luminosity program. It acts as an evaporator, absorbing and removing the increased thermal load from the higher radiation levels.  Quotable: “The right mindset unlocks solutions that technology alone cannot achieve,” Hemmeler said. “This isn’t just an incredible improvement ‒ it’s a fundamental reimagining of what’s possible. Thanks to CERN’s willingness to challenge the standard chiller-based cooling for data centers, we replaced mechanical cooling with only air and a little bit of water.”</t>
+          <t>The 2026 AHR Expo will be held in Las Vegas February 2–4, and components manufacturer NDL Industries is ready with a suite of products for CO2 (R744) refrigeration systems.
+The Vancouver-based company will showcase a “focused lineup of components” for high-pressure refrigeration systems, according to Paul Millard, National OEM Sales Manager. These include copper fittings, ball valves, check valves and NDL’s new three-way valves.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46001</v>
+        <v>46052</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hybrid dry coolers, manufactured by Swiss-based Jaeggi Hybridtechnologie (a subsidiary of Güntner), will provide all of the cooling for a CERN (European Organization for Nuclear Research) data center in Geneva, Switzerland, with an installed IT power capacity of 12MW. Ivan Hemmeler, Jaeggi’s Business Development Manager for Spain and Portugal, outlined the mechanical cooling-free system and its power usage effectiveness (PUE) in a presentation at the ATMOsphere (ATMO) Europe Summit 2025. ATMOsphere, publisher of NaturalRefrigerants.com, hosted the event, which was held November 24–25 in Padua, Italy.  PUE measures a data center’s energy efficiency by comparing the facility’s total power usage to that of the information technology equipment, including servers, storage and networks. A PUE of 1 represents theoretical perfection, with no power used for cooling and infrastructure. “By eliminating the chiller, we have removed the most energy-intensive component in traditional data center cooling,” Hemmeler said, with the hybrid dry cooler system providing a PUE of equal to or less than 1.15. “In addition, the technology uses 70% less water than conventional cooling towers, with just 0.379L [0.1gal] per kWh.” The design: A water-glycol loop transports the data center’s IT heat load directly to the hybrid dry coolers, where “massive double stacked” heat exchangers reject it using ambient air for the majority of the year in Geneva’s temperate climate. “The design is so simple, it becomes naturally resilient,” Hemmeler said.  In the event that temperatures rise to 40°C (104°F) during peak summer conditions, the heat exchanger coils are wetted, with the water fully recirculated. “A cascade design saves water while boosting cooling power, with smart controls optimizing operation based on climate and demand,” Hemmeler explained. Although the total system will be 12MW, currently just 8MW are installed. Of that, up to 4MW (1,137TR) of waste heat can be recovered and supplied to nearby CERN buildings for space heating. CERN, Jaeggi and Austrian refrigeration contractor Equans collaborated on the project.  What’s next: “With the units now installed, the real learning starts as we assess system behavior and refine its operation,” Hemmeler said.  Removing glycol is the next step to simplify the design, Hemmeler explained, adding that doing so could increase efficiency by 10‒20%. “We’ve successfully operated glycol-free data centers with Jaeggi [equipment] for 15 years,” he said. Recovering more waste heat from the system would also improve CERN’s PUE, he noted.  CERN and sustainability: CERN won the ATMO Europe 2025 Best-in-Sector/Industrial End User award for its use of a CO2 (R744)-based refrigeration system to cool its new high-luminosity Large Hadron Collider (LHC) program, scheduled to start operating in 2030.  CERN expects its new CO2 cooling system ‒ providing a combined capacity of 1.3MW (370TR) at its ATLAS and CMS particle detectors ‒ to reduce its greenhouse gas emissions by 40,000 metric tons of CO2e per year compared to synthetic alternatives. Swedish-based manufacturer SWEP developed Q185H, a new CO2 brazed plate heat exchanger, for CERN’s high-luminosity program. It acts as an evaporator, absorbing and removing the increased thermal load from the higher radiation levels.  Quotable: “The right mindset unlocks solutions that technology alone cannot achieve,” Hemmeler said. “This isn’t just an incredible improvement ‒ it’s a fundamental reimagining of what’s possible. Thanks to CERN’s willingness to challenge the standard chiller-based cooling for data centers, we replaced mechanical cooling with only air and a little bit of water.”</t>
+          <t>The 2026 AHR Expo will be held in Las Vegas February 2–4, and components manufacturer NDL Industries is ready with a suite of products for CO2 (R744) refrigeration systems.
+The Vancouver-based company will showcase a “focused lineup of components” for high-pressure refrigeration systems, according to Paul Millard, National OEM Sales Manager. These include copper fittings, ball valves, check valves and NDL’s new three-way valves. The company’s broad array of products for CO2 refrigeration systems is a reflection of its bullishness on the future of natural refrigerants in North America.
+“NDL sees continued momentum for CO2 refrigeration across the U.S. and Canadian markets,” Millard said.
+NaturalRefrigerants.com spoke with Millard to learn more about the products NDL will be exhibiting at AHR and the company’s outlook on natural refrigerants in the U.S.
+This interview has been edited for length and clarity.
+What CO2 products is NDL presenting at AHR 2026?
+Paul Millard: NDL Industries will be showcasing a focused lineup of components engineered specifically for high-pressure CO2 refrigeration systems at its booth #C2104.
+NDL’s CO2 ball valves and check valves are designed to withstand pressures up to 140bar [2,030psi]. NDL will also highlight its DN65 stainless steel CO2 ball valve, which is capable of handling pressures up to 130bar [1,885psi] and notable for its substantial size and suitability for large-scale CO2 applications.
+In addition, NDL will feature its CO2 copper fittings rated up to 130bar as well as CO2 service tees designed specifically for installing service valves with 10mm [3/8in] stainless steel stubs. These service tees reduce installation steps, eliminate the need for drilling or expanding fittings and ensure a precise fit for line sizes ranging from 1/2 to 2-1/8in [12.7 to 54mm].
+What message about CO2 or natural refrigerants will NDL be sharing with attendees?
+PM: NDL believes natural refrigerants represent the future of refrigeration, and CO2 plays a central role in that transition. At AHR, our message will focus on its commitment to supporting the market with reliable, high-quality components that are purpose-built for the unique demands of CO2 systems.
+By investing in products that meet the pressure, safety and performance requirements of modern CO2 refrigeration, NDL aims to help contractors, system designers and OEMs adopt natural refrigerants with confidence as the industry continues to evolve.
+“NDL believes natural refrigerants represent the future of refrigeration, and CO2 plays a central role in that transition.”
+Paul Millard, National OEM Sales Manager at NDL
+Does NDL have any new CO2 products under development?
+PM: NDL will be introducing its new CO2 three-way valves at AHR 2026. These valves are being developed specifically for high-pressure CO2 applications and represent an important expansion of NDL’s CO2 product portfolio.
+The introduction of these valves reflects our ongoing focus on addressing real world installation and system design needs within the CO2 refrigeration market while also offering a preview of what NDL is currently developing.
+How does NDL see the CO2 refrigeration sector in the U.S. evolving?
+PM: In the short term, including 2026, we expect rapid growth as aging refrigeration systems are replaced and regulatory pressures continue to favor natural refrigerants.
+In the long term, NDL anticipates steady and sustained adoption of CO2 technologies as familiarity increases, supply chains mature and system designs continue to improve. This long-term growth reinforces the need for durable, high-performance components designed specifically for CO2 applications.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-jaeggis-hybrid-dry-coolers-to-provide-cooling-for-12mw-cern-data-center-in-geneva/</t>
+          <t>https://naturalrefrigerants.com/news/ahr-2026-ndl-industries-details-the-co2-components-itll-be-exhibiting/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Enerblue Decarbonizes Railway Maintenance Hub with 900kW R290 Heat Pump System</t>
+          <t>Part 2: Why Penta Infra Chose Secon’s R290 Chillers for Its New Colocation Facility in Hamburg</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enerblue, an Italian HVAC manufacturer, has cut a major railway maintenance hub’s CO2e emissions by up to 90%, or roughly 672 metric tons, per year by replacing its gas heating unit with a 900kW (255.9TR) air-to-water propane (R290) heat pump system, according to the company. Through its German distributor, Kaut, Enerblue supplied and installed four of its Purplei R290 heat pumps connected in cascade to heat the 27,000m2 (290,630ft2) maintenance hub. The Purplei range offers heating capacities from 26 to 221kW (7.4 to 62.8TR), with outlet temperatures of up to 62°C (143.6°C) in −20°C (−4°F) ambient conditions. “The decision to heat the premises in a sustainable manner stemmed from the company’s desire to improve the site’s overall efficiency and reduce emissions,” Enerblue said. “After conducting technical assessments and tests on site, the solution was to install a natural refrigerant air-to-water heat pump system.” The setup: The hub’s underfloor heating enabled the technology transition, Enerblue explained, adding that it allowed lowering the delivery temperature from 75 to 55°C (167 to 131°F).  The cascade heat pump configuration enables dynamic power adjustment to ensure operational continuity, even during variable load periods, according to the manufacturer. A 1 million L (264,200gal) storage tank stabilizes the system and supports heat pump performance. A dual-fuel auxiliary boiler, capable of operating on hydrogen, provides supplemental heating in extreme weather conditions.  Additional measures: The existing photovoltaic array can power the heat pumps, according to Enerblue, with a building management system optimizing the new system’s performance.  Insulating the building and replacing the windows and doors improved the thermal energy efficiency of the maintenance facility.  Pressing forward: With its 10 years of experience manufacturing R290 and CO2 (R744) heat pumps and chillers, Enerblue continues to offer new programs and equipment.  In April the manufacturer started offering a five-year warranty exclusively for its natural refrigerant-based product portfolio. “This extended warranty is to make clear to our customers – and our customers’ customers – that we are really confident about our products,” Francesco Zanzo, Product Manager at Enerblue, told NaturalRefrigerants.com. In fall 2024 Enerblue introduced its Silver range of R290 chillers with cooling capacities of up to 768kW (218.3TR).  Quotable: “This project shows that adopting natural refrigerant heat pumps is a concrete, reliable solution for large-scale industrial applications,” Enerblue said. “It can guide companies towards more sustainable, efficient, future-oriented production models.” “This project shows that adopting natural refrigerant heat pumps is a concrete, reliable solution for large-scale industrial applications.” Enerblue</t>
+          <t>This is an excerpt from an article featured in ATMOsphere’s “Clean Cooling for Data Centers 2025” report, which can be downloaded here. ATMOsphere is the publisher of NaturalRefrigerants.com.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46000</v>
+        <v>46058</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Enerblue, an Italian HVAC manufacturer, has cut a major railway maintenance hub’s CO2e emissions by up to 90%, or roughly 672 metric tons, per year by replacing its gas heating unit with a 900kW (255.9TR) air-to-water propane (R290) heat pump system, according to the company. Through its German distributor, Kaut, Enerblue supplied and installed four of its Purplei R290 heat pumps connected in cascade to heat the 27,000m2 (290,630ft2) maintenance hub. The Purplei range offers heating capacities from 26 to 221kW (7.4 to 62.8TR), with outlet temperatures of up to 62°C (143.6°C) in −20°C (−4°F) ambient conditions. “The decision to heat the premises in a sustainable manner stemmed from the company’s desire to improve the site’s overall efficiency and reduce emissions,” Enerblue said. “After conducting technical assessments and tests on site, the solution was to install a natural refrigerant air-to-water heat pump system.” The setup: The hub’s underfloor heating enabled the technology transition, Enerblue explained, adding that it allowed lowering the delivery temperature from 75 to 55°C (167 to 131°F).  The cascade heat pump configuration enables dynamic power adjustment to ensure operational continuity, even during variable load periods, according to the manufacturer. A 1 million L (264,200gal) storage tank stabilizes the system and supports heat pump performance. A dual-fuel auxiliary boiler, capable of operating on hydrogen, provides supplemental heating in extreme weather conditions.  Additional measures: The existing photovoltaic array can power the heat pumps, according to Enerblue, with a building management system optimizing the new system’s performance.  Insulating the building and replacing the windows and doors improved the thermal energy efficiency of the maintenance facility.  Pressing forward: With its 10 years of experience manufacturing R290 and CO2 (R744) heat pumps and chillers, Enerblue continues to offer new programs and equipment.  In April the manufacturer started offering a five-year warranty exclusively for its natural refrigerant-based product portfolio. “This extended warranty is to make clear to our customers – and our customers’ customers – that we are really confident about our products,” Francesco Zanzo, Product Manager at Enerblue, told NaturalRefrigerants.com. In fall 2024 Enerblue introduced its Silver range of R290 chillers with cooling capacities of up to 768kW (218.3TR).  Quotable: “This project shows that adopting natural refrigerant heat pumps is a concrete, reliable solution for large-scale industrial applications,” Enerblue said. “It can guide companies towards more sustainable, efficient, future-oriented production models.” “This project shows that adopting natural refrigerant heat pumps is a concrete, reliable solution for large-scale industrial applications.” Enerblue</t>
+          <t>This is an excerpt from an article featured in ATMOsphere’s “Clean Cooling for Data Centers 2025” report, which can be downloaded here. ATMOsphere is the publisher of NaturalRefrigerants.com.
+In September 2023 Penta Infra broke ground on a new 4.4MW colocation facility in Hamburg located near the city’s airport. The Hamburg colocation facility opened in the first half of 2025 and boasts 2,500m2 (26,909ft2) of IT space.
+Six Secon air-cooled propane (R290) chillers were installed on the roof, each with a cooling capacity of 960kW (272TR) and a refrigerant charge of 38kg (84lbs) split across four separate refrigerant circuits. The water for the IT space is cooled to 20°C (68°F) and sent to computer room air-handlers, with the water returning to the chillers at a temperature of 32°C (89.6°F).
+The data center has been dubbed “Penta Infra HAM01” by Penta, with Ruben Uijtermerk, Mechanical Engineer at the company, stating that propane was chosen as a refrigerant because “it combines excellent thermodynamic efficiency with a very low GWP, providing high energy performance while maintaining environmental responsibility.”
+“Propane is particularly well-suited for medium-capacity applications like our Hamburg data center, offering reliable cooling performance with a proven safety record when installed with proper safety measures,” said Uijtermerk. “Secon’s extensive experience in implementing R290-based systems further ensures that safety and operational risks are minimized, adding confidence to this solution.”
+Read Part 1 Here
+Free cooling capabilities
+The chillers at the Penta Infra Hamburg data center feature a master–slave network, with two fully redundant and self-monitoring master controllers. They also come equipped with automatic transfer switches and uninterruptible power supplies for the controllers. Secon’s chillers include free cooling, but due to size limitations they cannot cover as much cooling capacity as the two dry coolers (there are plans to install two more). While separate units, the dry coolers are integrated into the chillers in terms of hydraulics and controls.
+Hamburg is located in northern Germany where summer temperatures range from 10 to 36°C (50 to 97°F), and winter temperatures range from −3 to 4°C (27 to 39°F). Thanks to the mild climate, the data center is able to use free cooling for a significant portion of the year. The power supply and control of the free coolers is managed by the chillers, which enables the full cooling capacity to be covered by free cooling. Pre-cooling mode starts at 27°C (80.6°F) and full free cooling is available from 16.5°C (61.7°F).
+“Up to 80% of the annual hours can be covered purely by free cooling,” Schadt said. “It’s a decisive factor in achieving a very low PUE value for the data center.”
+Pursuing a low PUE
+The PUE value for the facility is dictated by the German Energy Efficiency Act (EnEfG), which went into effect in November 2023 and requires all data centers with a connected load of 300kW or more to meet energy efficiency and waste heat requirements. Data centers commissioned before July 1, 2026, must have a PUE of ≤1.5 and a PUE of ≤1.3 by 2030.
+“We design according to the requirement in the EnEfG of an annual PUE of 1.2, meaning the hydrocarbon type chiller must be efficient enough to support this,” said Uijtermerk.
+The EnEfG also carries requirements to reuse waste heat, but as of 2025 there is no district heating network to connect to. Penta Infra HAM01 has two heat exchangers in the basement that enable it to connect to a district heating network, with the city and Penta Infra engaged in early discussions about a future district heating project.
+Uijtermerk said that in sites where district heating network connections are available, Penta sees “increased potential” in using reversible chillers, wherein heat is directly fed into the district heating network from the chiller; this would mitigate the need for dedicated heat pumps, increasing cost-effectiveness and maximizing the heat generating potential.
+Neither the EnEfG nor the EU F-gas Regulation broach the issues of HFOs or PFAS. However, Uijtermerk said that Penta more frequently sees natural refrigerants mentioned in client requests for information and requests for proposals.
+“There is increased awareness and appraisal by our clients for using natural refrigerants,” said Uijtermerk. “Penta believes that, if practically possible, hydrocarbons are the better choice over synthetic refrigerants.”</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/enerblue-decarbonizes-railway-maintenance-hub-with-900kw-r290-heat-pump-system/</t>
+          <t>https://naturalrefrigerants.com/news/part-2-why-penta-infra-chose-secons-r290-chillers-for-its-new-colocation-facility-in-hamburg/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>New York Grassroots Group Leads Successful Refrigerant Recycling Drives</t>
+          <t>ATMO Europe: Unic Air Set to Launch AHU with CO2 Heat Pump Delivering Space Heating and Cooling</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Given their outsize impact of f-gases on the environment, “my belief is that appliances [with f-gas refrigerants] are the most important thing a person could ever recycle,” said Michael Helme, Co-Founder and Lead Volunteer of New Yorkers for Cool Refrigerant Management (NY4Cool). Formed in 2020, NY4Cool is a grassroots group dedicated to preventing refrigerant pollution through community action such as appliance recycling drives, operating mostly in Orange and Ulster Counties in New York State, just north of New York City. The volunteer group is one of the few in the U.S. – if not the only one – with a focus on preventing emissions of fluorinated refrigerants from home appliances like air conditioners, refrigerators and dehumidifiers. (This does not include home heat pumps and split or ducted AC systems, for which refrigerants must be reclaimed by a certified technician on site.) NY4Cool also advocates for faster adoption of natural refrigerant-based HVAC&amp;R systems and equipment. “If you burn a pound of gasoline, it will create 3.25 pounds of carbon dioxide,” Helme said at a press conference in 2024. “If you release a pound of R410A into the atmosphere, it will act like more than 4,000 pounds of carbon dioxide [equivalent] over the next 20 years – and a single air conditioner could have a pound or two of R410A.” On November 6, Helme, his NY4Cool group and six New York municipalities received the 2025 “Building Bridges Award” from the Hudson Valley Regional Council (HVRC) for their work in collecting and recycling hundreds of old refrigerant appliances via an initiative called the “Coolest Recycling Drive.” Suzanne Hagell, Chief, GHG Mitigation Office, New York State Department of Environmental Conservation (DEC), presented the award to Helme and the municipalities, which include the City of Kingston, Town of Chester, Town of Warwick, Town of New Paltz, Village of New Paltz and Village of Woodbury. Underscoring the impact that refrigerant recycling can have, Helme noted at the awards ceremony that the town of New Paltz alone, which typically generates 400 metric tons of annual emissions from its municipal buildings, prevented the emissions of 160 metric tons of CO2e as a result of the 2025 appliance drive. “It was so easy to do,” he said. “We had 10 volunteers who worked at three drop-off events, each four hours long, and we spent just a few hundred dollars.” End-of-life emissions In the U.S., the Clean Air Act prohibits individuals from intentionally venting ozone-depleting refrigerants and HFCs while maintaining, servicing, repairing or disposing of air-conditioning or refrigeration equipment. However, this regulation, as well as similar state rules, are difficult to enforce. End-of-life emissions of HCFC and HFC refrigerants from retired equipment that could have been collected are estimated to account for 75 to 80 million metric tons of CO2e annually in the U.S., equivalent to emissions from 16 million cars, according to a 2019 report by the Environmental Investigation Agency (EIA). On top of that, Helme noted, there is a thriving international market in shipping old appliances to Asian countries, China in particular, where the refrigerant is likely vented. But as a result of the U.S. AIM Act, which has devised a phasedown schedule for HFC production and import, the amount of reclaimed HFCs has grown from 5 million pounds (2.3 million kilograms) in 2017 to 12 million pounds (5.4 million kilograms) in 2024, according to the EPA. Beginning January 1, 2029, the servicing and/or repair of HFC-containing supermarket systems, refrigerated transport and automatic commercial ice makers must be done with reclaimed HFCs. Recipients of 2025 Building Bridges Award from the Hudson Valley (New York) Regional Council (HVRC), from left: Mayor Andrew Giacomazza and Lisa Marie Hintze, Village of Woodbury; Bill Greene, Town of Chester; Julie Noble, City of Kingston; HVRC’s Executive Director Carla Castillo; Melissa Apuzzo, Town of Warwick; Janelle Peotter and Yvonne Posey, Town of New Paltz; Mark Varian, Village of New Paltz; and Michael Helme, Town of Warwick and New Yorkers for Cool Refrigerant Management (NY4Cool); the award was presented by Suzanne Hagell, New York State DEC Office of Climate Change, far right. Volunteers in the NY4Cool appliance recycling drives often wear sunglasses, which refer to the group’s logo. Image from hudsonvalleyregionalcouncil.org. While local recycling transfer stations accept refrigerant-bearing appliances, they typically charge a fee and are not necessarily conveniently located; moreover, they usually don’t prioritize refrigerant reclaim. Helme came up with the idea of recycling drives to make the appliance drop-off process free and local during specified times of the year (typically the spring), thereby achieving more f-gas recovery. The NY4Cool group emerged from a refrigerant management working group led by Sustainable Hudson Valley, a nonprofit under which NY4Cool still operates. The interest in refrigerant management was inspired by Project Drawdown, a major climate change initiative that identified refrigerant emissions reduction as one of the most important greenhouse gas remediation measures. “A few of us wanted to keep discussing the topic of refrigerants,” said Helme, who formerly worked in support staff for a large law firm and translated Chinese medicine books on the side. “I didn’t have any background in [refrigerants]. I don’t know why I stuck to that group, but it somehow kind of appealed to me. And then it just seemed like we could really be doing something here.” NY4Cool now has a mailing list of about 50 people, including professionals in HVAC&amp;R and citizen activists like Helme. Christina Starr, Senior Manager, Climate for U.S. branch of the EIA, has been a major contributor to the group. Earth Week launch Helme launched the first Coolest Reycling Driven in 2023 during a two-week period encompassing Earth Week (April 14 to 22) in Warwick, New York, where he lives, in concert with a local nonprofit environmental group,  Sustainable Warwick. The groups hired a refrigerant reclaimer, Interstate Refrigerant Recovery Inc. (IRRI), which charged $9 apiece. Compared to the inventory of appliances received, the recovered refrigerants totalled approximately 80% of the CO2e in the appliances, he said. Helme publicized the drive through Sustainable Warwick and the town of Warwick, drawing from a diverse population. “The people who brought their appliances were not all the usual suspects who usually show up at the Sustainable Warwick events,” he said. “It didn’t matter their political stripe or economic status; it was just anybody with a piece of junk they wanted to get rid of.” That initial drive received about 130 appliances and four refrigerant tanks. It prevented the equivalent of nearly 500,000lbs (226,796kg) of CO2e emissions (based on a 20-year GWP,  the standard used in New York) and sent more than 4,000lbs (1,814kg) of metal for recycling, all for a net cost of about $900, according to the NY4Cool estimates. “When they prevent another 100,000 pounds of CO2 equivalent [emissions], people go home feeling really good.” Michael Helme, Lead Volunteer, New Yorkers for Cool Refrigerant Management In 2024, Hudson Technologies, a refrigerant reclamation company based in Woodcliff Lake, New Jersey, offered to provide refrigerant recovery work at no charge for the 2024 Cooling Recycling Drive. This enabled the NY4Cool, Sustainable Warwick and Sustainable Hudson Valley, to team up with numerous community organizations and hold an expanded Coolest Recycling Drive in the spring in Orange and Ulster counties. The drive collected 500 appliances, said Helme. In October 2024 another collection effort was held in Woodbury, New York, and surrounding communities, which netted 26 air conditioners, 16 refrigerators and seven dehumidifiers, according to NY4Cool. In 2025, the spring recycling drive in the six award-winning communities in Orange and Ulster Counties collected about 435 appliances; assuming a conservative recovery rate of 50% of the refrigerant, this accounts for about 335 metric tons of CO2e, equivalent to driving 78 gas-powered automobiles for one year, said NY4Cool. For the reclamation work, NY4Cool hired JGS Recycling &amp; Hauling, which charged $3 apiece for appliances (typically ACs) hauled away for scrap, and $7 apiece for other appliances. Helme has collaborated with the local Lions Club to publicize and support the recycling drives, resulting in a spike of appliance drop-offs. “That’s just been very gratifying, working with the Lions Club,” he said. NY4Cool has also partnered with local Climate Smart Community groups, part of a program started by the New York State DEC for municipal governments to promote climate-related mitigation and adaptation efforts. Appliance recycling drives earn these communities recognition “points” under the general educational umbrella toward getting certified as a Climate Smart Community by the state, said Eleanor Peck, Deputy Executive Director for the HVRC. Incentivizing reclaim Because recycling transfer stations often don’t prioritize refrigerant-bearing appliances, Helme plans to lobby for state funding that would incentivize them to do reclamation work. “Then the refrigerant recovery work is all paid for, and all they have to do is line the appliances up and get the scrap metal money at the end,” he said. “It becomes a cash-flow positive thing for the transfer station. So they want to do as much of it as they can.” NY4Cool also supports the eventual adoption in New York of an extended producer responsibility program for refrigerants that will make recovery, reclamation and destruction a standard practice overseen by the producers of refrigerants and equipment. A few of the appliances dropped off at the 2025 Coolest Recycling Drive organized by New Yorkers for Cool Refrigerant Management. Image from www.ny4cool.org.  While grassroots drives like those implemented by NY4Cool are rare outside of New York, the group has posted a recycling guide on its website for others to follow. ‘I’d like to see it take off, but it hasn’t,” said Helme. He finds that volunteers enjoy participating in appliance-recycling drives. “People are so frustrated about what they can do about the climate crisis,” he said. “But when they prevent another 100,000 pounds of CO2 equivalent [emissions], people go home feeling really good. I wish more people had that feeling.”</t>
+          <t>In spring 2026 Danish HVAC manufacturer Unic Air will launch COOLHEAT, a bespoke air handling unit (AHU) that delivers space heating and cooling via a CO2 (R744) heat pump. The self-contained unit was developed in collaboration with the Danish Technological Institute (DTI).
+Christian Heerup, Business Manager of Refrigeration at DTI, along with Allan Kjær, Head of Research and Development at Unic Air, outlined the unit’s development and testing in a presentation at the ATMOsphere (ATMO) Europe Summit 2025.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46006</v>
+        <v>46056</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Given their outsize impact of f-gases on the environment, “my belief is that appliances [with f-gas refrigerants] are the most important thing a person could ever recycle,” said Michael Helme, Co-Founder and Lead Volunteer of New Yorkers for Cool Refrigerant Management (NY4Cool). Formed in 2020, NY4Cool is a grassroots group dedicated to preventing refrigerant pollution through community action such as appliance recycling drives, operating mostly in Orange and Ulster Counties in New York State, just north of New York City. The volunteer group is one of the few in the U.S. – if not the only one – with a focus on preventing emissions of fluorinated refrigerants from home appliances like air conditioners, refrigerators and dehumidifiers. (This does not include home heat pumps and split or ducted AC systems, for which refrigerants must be reclaimed by a certified technician on site.) NY4Cool also advocates for faster adoption of natural refrigerant-based HVAC&amp;R systems and equipment. “If you burn a pound of gasoline, it will create 3.25 pounds of carbon dioxide,” Helme said at a press conference in 2024. “If you release a pound of R410A into the atmosphere, it will act like more than 4,000 pounds of carbon dioxide [equivalent] over the next 20 years – and a single air conditioner could have a pound or two of R410A.” On November 6, Helme, his NY4Cool group and six New York municipalities received the 2025 “Building Bridges Award” from the Hudson Valley Regional Council (HVRC) for their work in collecting and recycling hundreds of old refrigerant appliances via an initiative called the “Coolest Recycling Drive.” Suzanne Hagell, Chief, GHG Mitigation Office, New York State Department of Environmental Conservation (DEC), presented the award to Helme and the municipalities, which include the City of Kingston, Town of Chester, Town of Warwick, Town of New Paltz, Village of New Paltz and Village of Woodbury. Underscoring the impact that refrigerant recycling can have, Helme noted at the awards ceremony that the town of New Paltz alone, which typically generates 400 metric tons of annual emissions from its municipal buildings, prevented the emissions of 160 metric tons of CO2e as a result of the 2025 appliance drive. “It was so easy to do,” he said. “We had 10 volunteers who worked at three drop-off events, each four hours long, and we spent just a few hundred dollars.” End-of-life emissions In the U.S., the Clean Air Act prohibits individuals from intentionally venting ozone-depleting refrigerants and HFCs while maintaining, servicing, repairing or disposing of air-conditioning or refrigeration equipment. However, this regulation, as well as similar state rules, are difficult to enforce. End-of-life emissions of HCFC and HFC refrigerants from retired equipment that could have been collected are estimated to account for 75 to 80 million metric tons of CO2e annually in the U.S., equivalent to emissions from 16 million cars, according to a 2019 report by the Environmental Investigation Agency (EIA). On top of that, Helme noted, there is a thriving international market in shipping old appliances to Asian countries, China in particular, where the refrigerant is likely vented. But as a result of the U.S. AIM Act, which has devised a phasedown schedule for HFC production and import, the amount of reclaimed HFCs has grown from 5 million pounds (2.3 million kilograms) in 2017 to 12 million pounds (5.4 million kilograms) in 2024, according to the EPA. Beginning January 1, 2029, the servicing and/or repair of HFC-containing supermarket systems, refrigerated transport and automatic commercial ice makers must be done with reclaimed HFCs. Recipients of 2025 Building Bridges Award from the Hudson Valley (New York) Regional Council (HVRC), from left: Mayor Andrew Giacomazza and Lisa Marie Hintze, Village of Woodbury; Bill Greene, Town of Chester; Julie Noble, City of Kingston; HVRC’s Executive Director Carla Castillo; Melissa Apuzzo, Town of Warwick; Janelle Peotter and Yvonne Posey, Town of New Paltz; Mark Varian, Village of New Paltz; and Michael Helme, Town of Warwick and New Yorkers for Cool Refrigerant Management (NY4Cool); the award was presented by Suzanne Hagell, New York State DEC Office of Climate Change, far right. Volunteers in the NY4Cool appliance recycling drives often wear sunglasses, which refer to the group’s logo. Image from hudsonvalleyregionalcouncil.org. While local recycling transfer stations accept refrigerant-bearing appliances, they typically charge a fee and are not necessarily conveniently located; moreover, they usually don’t prioritize refrigerant reclaim. Helme came up with the idea of recycling drives to make the appliance drop-off process free and local during specified times of the year (typically the spring), thereby achieving more f-gas recovery. The NY4Cool group emerged from a refrigerant management working group led by Sustainable Hudson Valley, a nonprofit under which NY4Cool still operates. The interest in refrigerant management was inspired by Project Drawdown, a major climate change initiative that identified refrigerant emissions reduction as one of the most important greenhouse gas remediation measures. “A few of us wanted to keep discussing the topic of refrigerants,” said Helme, who formerly worked in support staff for a large law firm and translated Chinese medicine books on the side. “I didn’t have any background in [refrigerants]. I don’t know why I stuck to that group, but it somehow kind of appealed to me. And then it just seemed like we could really be doing something here.” NY4Cool now has a mailing list of about 50 people, including professionals in HVAC&amp;R and citizen activists like Helme. Christina Starr, Senior Manager, Climate for U.S. branch of the EIA, has been a major contributor to the group. Earth Week launch Helme launched the first Coolest Reycling Driven in 2023 during a two-week period encompassing Earth Week (April 14 to 22) in Warwick, New York, where he lives, in concert with a local nonprofit environmental group,  Sustainable Warwick. The groups hired a refrigerant reclaimer, Interstate Refrigerant Recovery Inc. (IRRI), which charged $9 apiece. Compared to the inventory of appliances received, the recovered refrigerants totalled approximately 80% of the CO2e in the appliances, he said. Helme publicized the drive through Sustainable Warwick and the town of Warwick, drawing from a diverse population. “The people who brought their appliances were not all the usual suspects who usually show up at the Sustainable Warwick events,” he said. “It didn’t matter their political stripe or economic status; it was just anybody with a piece of junk they wanted to get rid of.” That initial drive received about 130 appliances and four refrigerant tanks. It prevented the equivalent of nearly 500,000lbs (226,796kg) of CO2e emissions (based on a 20-year GWP,  the standard used in New York) and sent more than 4,000lbs (1,814kg) of metal for recycling, all for a net cost of about $900, according to the NY4Cool estimates. “When they prevent another 100,000 pounds of CO2 equivalent [emissions], people go home feeling really good.” Michael Helme, Lead Volunteer, New Yorkers for Cool Refrigerant Management In 2024, Hudson Technologies, a refrigerant reclamation company based in Woodcliff Lake, New Jersey, offered to provide refrigerant recovery work at no charge for the 2024 Cooling Recycling Drive. This enabled the NY4Cool, Sustainable Warwick and Sustainable Hudson Valley, to team up with numerous community organizations and hold an expanded Coolest Recycling Drive in the spring in Orange and Ulster counties. The drive collected 500 appliances, said Helme. In October 2024 another collection effort was held in Woodbury, New York, and surrounding communities, which netted 26 air conditioners, 16 refrigerators and seven dehumidifiers, according to NY4Cool. In 2025, the spring recycling drive in the six award-winning communities in Orange and Ulster Counties collected about 435 appliances; assuming a conservative recovery rate of 50% of the refrigerant, this accounts for about 335 metric tons of CO2e, equivalent to driving 78 gas-powered automobiles for one year, said NY4Cool. For the reclamation work, NY4Cool hired JGS Recycling &amp; Hauling, which charged $3 apiece for appliances (typically ACs) hauled away for scrap, and $7 apiece for other appliances. Helme has collaborated with the local Lions Club to publicize and support the recycling drives, resulting in a spike of appliance drop-offs. “That’s just been very gratifying, working with the Lions Club,” he said. NY4Cool has also partnered with local Climate Smart Community groups, part of a program started by the New York State DEC for municipal governments to promote climate-related mitigation and adaptation efforts. Appliance recycling drives earn these communities recognition “points” under the general educational umbrella toward getting certified as a Climate Smart Community by the state, said Eleanor Peck, Deputy Executive Director for the HVRC. Incentivizing reclaim Because recycling transfer stations often don’t prioritize refrigerant-bearing appliances, Helme plans to lobby for state funding that would incentivize them to do reclamation work. “Then the refrigerant recovery work is all paid for, and all they have to do is line the appliances up and get the scrap metal money at the end,” he said. “It becomes a cash-flow positive thing for the transfer station. So they want to do as much of it as they can.” NY4Cool also supports the eventual adoption in New York of an extended producer responsibility program for refrigerants that will make recovery, reclamation and destruction a standard practice overseen by the producers of refrigerants and equipment. A few of the appliances dropped off at the 2025 Coolest Recycling Drive organized by New Yorkers for Cool Refrigerant Management. Image from www.ny4cool.org.  While grassroots drives like those implemented by NY4Cool are rare outside of New York, the group has posted a recycling guide on its website for others to follow. ‘I’d like to see it take off, but it hasn’t,” said Helme. He finds that volunteers enjoy participating in appliance-recycling drives. “People are so frustrated about what they can do about the climate crisis,” he said. “But when they prevent another 100,000 pounds of CO2 equivalent [emissions], people go home feeling really good. I wish more people had that feeling.”</t>
+          <t>In spring 2026 Danish HVAC manufacturer Unic Air will launch COOLHEAT, a bespoke air handling unit (AHU) that delivers space heating and cooling via a CO2 (R744) heat pump. The self-contained unit was developed in collaboration with the Danish Technological Institute (DTI).
+Christian Heerup, Business Manager of Refrigeration at DTI, along with Allan Kjær, Head of Research and Development at Unic Air, outlined the unit’s development and testing in a presentation at the ATMOsphere (ATMO) Europe Summit 2025. The event, organized by ATMOsphere, was held November 24–25 in Padua, Italy. ATMOsphere is the publisher of NaturalRefrigerants.com.
+“We have seven years of experience cooling with CO2,” Kjær said, adding that Unic Air has more than 250 CO2 HVAC units operating in Denmark. “However, we see a bigger and bigger need for adding heating.”
+Unic Air and DTI initiated their collaboration in 2021 with the goal of producing an “HFC-free alternative for conditioning fresh air,” according to Heerup. By 2023, the partnership had a prototype in development. In summer 2024 DTI conducted laboratory testing, followed by Unic Air’s installing the unit in its office building for demonstration.
+Details/performance: The design incorporates two inverter-driven CO2 Dorin compressors, with a rotating heat exchanger covering the majority of the load, according to Heerup.
+The unit shares components across its circuits while featuring separate heating and cooling coils, integrated into a single block handling both supply and exhaust air. U.K.–based 3T supplies the coils, while Italian-based Carel provides the controls.
+Testing in the Unic Air office building gave a COP of 3.7 in ambient conditions ranging from 19 to 23°C (66 to 73°F) and a COP of 2.2 in temperatures over 27°C (81°F). In temperatures below −5°C (23°F), it provided a COP of 3.2, with defrosting taking 5‒10% of the COP.
+“It’s market–ready and suitable for northern climates,” Heerup said, adding that it costs roughly 20% more than a comparable HFC-based AHU.
+Overcoming challenges: Conditions in Denmark require seven times more airflow in warm months compared to cold ones, making it difficult to maintain stable operation and high COPs in the operating extremes.
+DTI optimized one of the compressors for summer loads and one for low–frequency/part–load winter operation.
+Increasing the superheat setpoint from 7 to 10K (7 to 10°C/12.6 to 18°F) resolved issues with cold compressor operation and foaming oil, which increased the COP from 2.2 to 3.1. The partnership also replaced the evaporator coil in the exhaust air to support even frosting.
+Potential upgrade: The next generation design by DTI and Unic Air for an AHU using a CO2 heat pump includes coils in both parallel and counter flow, a four-way changeover valve, an integrated ejector and an internal heat exchanger/oil rectifier. Heerup also suggested evaluating permanent magnetic motor compressors.
+The team completed a high ambient temperature design for a potential unit in May 2025, but ran out of funds to build it with the project terminating in February 2026, according to Heerup.
+Potential options: A couple of other European manufacturers have AHUs using CO2 refrigerant in various stages of development.
+German HVAC designer and manufacturer Menerga showcased a prototype of an AHU with a CO2 heat pump for public-swimming-pool dehumidification at ISH 2025, with 20kW (5.7TR) of cooling capacity and 25kW (7.1TR) of heating. It produces outlet water temperatures of up to 65°C (149°F).
+U.K.-based heat pump manufacturer Clade Engineering Systems offers a combined AHU and heat pump using a direct expansion CO2 heat transfer coil. The modular unit comes in 50, 100, 125, and 150kW (14.2, 28.4, 35.5 and 42.7TR) capacities.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/new-york-grassroots-group-leads-successful-refrigerant-recycling-drives/</t>
+          <t>https://naturalrefrigerants.com/news/atmo-europe-unic-air-set-to-launch-ahu-with-co2-heat-pump-delivering-heating-and-cooling/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>German Produce Wholesaler Replaces R404A Refrigeration With Frigotec R290 Chiller</t>
+          <t>Brazil HVAC&amp;R Association Presents Proposed Strategy for First Phase of National HFC Reduction Program</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>German produce wholesaler Fruchthof Northeim has replaced its R404A refrigeration system with a propane (R290) chiller with a 61.8kW (17.6TR) cooling capacity, produced by German refrigeration manufacturer Frigotec. The March retrofit highlights Frigotec’s first deployment of its new R290 FrigoNatura series. The line incorporates German Bitzer Ecoline Pro reciprocating compressors manufactured for use with hydrocarbon refrigerants. “Due to the electrical demand of the fruit processor’s existing refrigeration system in peak summer months, Frigotec placed emphasis on selecting energy–efficient system components and optimizing control technology,” Bitzer said. “Highlights [of the installation] include our electronic compressor control IQ MODULE CM-RC-02 and the Siemens MLV702 magnetic expansion valve, which enables fast and precise response time.” Fruchthof Northeim chose a propane refrigeration system based on several factors, according to Bitzer, including the phase out of fluorinated refrigerants by the EU’s F-gas Regulation, reduced energy consumption and operating costs and the ability to improve its CO2e footprint. The setup: The chiller, installed outside the Northeim facility, is divided between two refrigeration circuits, each with a 4-cylinder compressor.  A chilled secondary ethylene glycol loop, circulated by variable speed pumps, maintains two cold-storage rooms with a combined area of 167m2 (1,800ft2) at a constant temperature of 4°C (39.2°F). On the brine side, the system connects to two 2,500L (660gal) buffer tanks, located in a separate machine room. Heat is rejected through air-cooled condensers, while recovered heat from the R290 refrigeration system will later be used to provide space heating for the facility once all cold-storage rooms have been modernized, according to Bitzer.  Safety and control: “The fruit market’s new refrigeration system meets the highest safety standards for operation with propane and offers efficient part-load capability,” Bitzer said.  The use of Bitzer’s ECOLINE PRO series, which complies with the EU’s explosion-prevention requirements specified in EN 1127-1, removes the need for an ATEX-classified area around the compressors. The installation is further safeguarded by a gas-detection sensor, exhaust fan and warning light/siren. Bitzer’s mechanical capacity control system, VARISTEP, allows a single compressor to operate at 50%. If one compressor is off at the Northeim facility and the other one operates at 50%, the total cooling capacity of the liquid chiller can be reduced to 25% or 15.5kW (4.4TR), which provides seasonal flexibility, Bitzer explained.  R290 chiller line: Frigotec offers its FrigoNatura product range in three sizes covering cooling capacities from 25 to over 400kW (7.1 to over 113.7TR) for commercial and industrial chiller, brine chiller and heat pump applications.  Bitzer’s Ecoline Pro series compressors, which offer refrigeration capacities from 0.9 to 110kW (0.26 to 31.3TR) and heating capacities from 2 to 238kW (0.57 to 64.8TR), come in models featuring 2, 4, 6 or 8 cylinders. In June Frigotec commissioned the largest version of its new R290 chiller with a cooling capacity of more than 400kW in a jam manufacturing plant, according to authorized Frigotec signatory Lucas Einenkel.  Quotable: “The project with the Northeim fruit market was a successful start for our FrigoNatura series,” Einenkel said. “Using the IQ MODULE provides detailed compressor [and] system data, which gives insight into the operating behavior and improves overall system reliability.”  “The fruit market’s new refrigeration system meets the highest safety standards for operation with propane and offers efficient part-load capability.” Bitzer</t>
+          <t>The Brazilian Association of Refrigeration, Air Conditioning, Ventilation and Heating (ABRAVA) has presented a proposed strategy for the first phase of Brazil’s national program to reduce the consumption of HFCs.
+The first phase of the Brazilian Program for Reducing the Consumption of HFCs (HFCs Program) will run from 2027 to 2032 and aims to cut national HFC consumption by 10% by 2029 – equivalent to approximately 7.3 million metric tons of CO2e.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46003</v>
+        <v>46059</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>German produce wholesaler Fruchthof Northeim has replaced its R404A refrigeration system with a propane (R290) chiller with a 61.8kW (17.6TR) cooling capacity, produced by German refrigeration manufacturer Frigotec. The March retrofit highlights Frigotec’s first deployment of its new R290 FrigoNatura series. The line incorporates German Bitzer Ecoline Pro reciprocating compressors manufactured for use with hydrocarbon refrigerants. “Due to the electrical demand of the fruit processor’s existing refrigeration system in peak summer months, Frigotec placed emphasis on selecting energy–efficient system components and optimizing control technology,” Bitzer said. “Highlights [of the installation] include our electronic compressor control IQ MODULE CM-RC-02 and the Siemens MLV702 magnetic expansion valve, which enables fast and precise response time.” Fruchthof Northeim chose a propane refrigeration system based on several factors, according to Bitzer, including the phase out of fluorinated refrigerants by the EU’s F-gas Regulation, reduced energy consumption and operating costs and the ability to improve its CO2e footprint. The setup: The chiller, installed outside the Northeim facility, is divided between two refrigeration circuits, each with a 4-cylinder compressor.  A chilled secondary ethylene glycol loop, circulated by variable speed pumps, maintains two cold-storage rooms with a combined area of 167m2 (1,800ft2) at a constant temperature of 4°C (39.2°F). On the brine side, the system connects to two 2,500L (660gal) buffer tanks, located in a separate machine room. Heat is rejected through air-cooled condensers, while recovered heat from the R290 refrigeration system will later be used to provide space heating for the facility once all cold-storage rooms have been modernized, according to Bitzer.  Safety and control: “The fruit market’s new refrigeration system meets the highest safety standards for operation with propane and offers efficient part-load capability,” Bitzer said.  The use of Bitzer’s ECOLINE PRO series, which complies with the EU’s explosion-prevention requirements specified in EN 1127-1, removes the need for an ATEX-classified area around the compressors. The installation is further safeguarded by a gas-detection sensor, exhaust fan and warning light/siren. Bitzer’s mechanical capacity control system, VARISTEP, allows a single compressor to operate at 50%. If one compressor is off at the Northeim facility and the other one operates at 50%, the total cooling capacity of the liquid chiller can be reduced to 25% or 15.5kW (4.4TR), which provides seasonal flexibility, Bitzer explained.  R290 chiller line: Frigotec offers its FrigoNatura product range in three sizes covering cooling capacities from 25 to over 400kW (7.1 to over 113.7TR) for commercial and industrial chiller, brine chiller and heat pump applications.  Bitzer’s Ecoline Pro series compressors, which offer refrigeration capacities from 0.9 to 110kW (0.26 to 31.3TR) and heating capacities from 2 to 238kW (0.57 to 64.8TR), come in models featuring 2, 4, 6 or 8 cylinders. In June Frigotec commissioned the largest version of its new R290 chiller with a cooling capacity of more than 400kW in a jam manufacturing plant, according to authorized Frigotec signatory Lucas Einenkel.  Quotable: “The project with the Northeim fruit market was a successful start for our FrigoNatura series,” Einenkel said. “Using the IQ MODULE provides detailed compressor [and] system data, which gives insight into the operating behavior and improves overall system reliability.”  “The fruit market’s new refrigeration system meets the highest safety standards for operation with propane and offers efficient part-load capability.” Bitzer</t>
+          <t>The Brazilian Association of Refrigeration, Air Conditioning, Ventilation and Heating (ABRAVA) has presented a proposed strategy for the first phase of Brazil’s national program to reduce the consumption of HFCs.
+The first phase of the Brazilian Program for Reducing the Consumption of HFCs (HFCs Program) will run from 2027 to 2032 and aims to cut national HFC consumption by 10% by 2029 – equivalent to approximately 7.3 million metric tons of CO2e. This target aligns with Brazil’s commitments under the Kigali Amendment to the Montreal Protocol, which the country ratified in October 2022.
+The proposed strategy centers on a package of regulatory measures designed to support Brazil’s transition to low-GWP and energy-efficient refrigerants across multiple sectors, including natural refrigerant training for technicians. In addition to commercial refrigeration and air-conditioning, the strategy covers mobile air-conditioning (MAC), data centers, industrial refrigeration and heat pumps.
+“The active participation of different sectors is essential to ensure that public policies reflect the real needs of the market and society,” said Frank Amorim, Technical Representative of Brazil’s Ministry of Environment and Climate Change (MMA). “More than a set of actions, this is a comprehensive study on the consumption of these gases in various sectors in Brazil, offering a solid basis for the technological and energy transition.”
+The proposed strategy was presented at a meeting held in São Paulo on December 1, organized by the MMA in partnership with the United Nations Development Programme (UNDP), the United Nations Industrial Development Organization (UNIDO) and Germany’s development agency, the GIZ (German Agency for International Cooperation).
+The MMA is accepting public feedback on the proposed strategy for the first phase of the HFCs Program through December 27.
+“More than a set of actions, this is a comprehensive study on the consumption of these gases in various sectors in Brazil, offering a solid basis for the technological and energy transition.”
+Frank Amorim, Technical Representative of Brazil’s Ministry of Environment and Climate Change
+Curbing rising consumption
+Without additional action, Brazil’s HFC consumption could reach 55 million metric tons of CO2e by 2035, surpassing its allocated limit of 51 million metric tons under the Kigali Amendment, according to Ana Paula Leal, Project Coordinator for UNDP. The HFCs Program is intended to ensure compliance with these international obligations.
+Proposed measures include establishing maximum GWP limits by equipment type and/or sector, banning the use of R134a and R410A in residential refrigerators and air conditioners starting in 2029 and implementing mandatory energy-efficiency labeling for refrigeration and air-conditioning equipment. The strategy also highlights the need for sector-specific policies for supermarkets to support a safe and economically viable transition to low-GWP and energy-efficient refrigerants, as well as the internalization of international HVAC&amp;R standards.
+Capacity building is also a core component of the proposed strategy, with plans to launch a Qualification, Certification and Registration project, which will develop and test a system for expanding and upskilling Brazil’s HVAC&amp;R workforce. The strategy also includes additional technician training focused on the safe and efficient use of natural refrigerants, as well as a project for mandatory refrigerant handling and maintenance practices in the MAC sector.
+These training efforts will build on progress achieved under Brazil’s HCFC Elimination Program (PBH), according to Stefanie von Heinemann, Consultant and Project Manager for the GIZ.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/german-produce-wholesaler-replaces-r404a-refrigeration-with-61-8kw-frigotec-r290-liquid-chiller/</t>
+          <t>https://naturalrefrigerants.com/news/brazil-hvacr-association-presents-proposed-strategy-for-first-phase-of-national-hfc-reduction-program/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sanhua to Offer ‘Complete Packages’ of Components for CO2 and Propane Commercial Refrigeration Systems</t>
+          <t>Duke University Researchers Study Potential Link Between PFAS, Including TFA, and Thyroid Dysfunction in Firefighters</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Components manufacturer Sanhua has announced that it will begin supplying “complete packages” of “coordinated and compatible components” for commercial refrigeration systems using propane (R290) and CO2 (R744) refrigerants. The product packages are part of the company’s 2025–2030 roadmap, which is oriented around natural refrigerants and integrated component packages. Federico Bisco, Technical Director of Sanhua Europe, said the company “has deliberately chosen not to present itself as a manufacturer of finished systems.” Rather, its goal is to help manufacturers reduce the complexity of sourcing components, lower costs through bulk purchases and simplify approving and testing systems. Sanhua is making its product packages available for three types of commercial refrigeration systems: propane plug-ins, propane waterloops and CO2 condensing units. The propane plug-in package: Sanhua said it’s already able to cover “more than 90%” of the components needed for propane plug-in applications.  A product package for propane plug-ins includes filters, solenoid valves, thermostatic expansion valve, electronic expansion valve, exchangers, taps, sensors, electronic controllers, inverters and thermostats. “Package integration allows OEMs to reduce the bill of materials and facilitate system approval,” Sanhua said.  The waterloop package: Sanhua offers three types of product packages for R290 waterloops.  Basic (with mechanical valve), smart (with electronic valve and sensors) and plus (with inverter and digital controller). The product packages are designed for applications where compactness and flexibility are crucial, Sanhua said, and are a fit for small-format grocery stores, convenience stores and retrofits of existing systems.  The CO2 condensing unit package: Sanhua’s product package for CO2 condensing units will include “all critical components,” including pulse expansion valves, smart sensors, heat exchangers, controllers and safety valves. The product package is expected to be available by the end of 2026, and Sanhua is initially targeting CO2 condensing units under 40kW (11.3TR), although it plans to expand the product package to transcritical racks with a capacity of up to 100kW (28.4TR).  “The main challenge is to make CO2 condensing units competitive with HFO solutions,” Bisco said. “Costs remain two to three times higher, but increased volumes and standardized designs are expected to narrow the gap.”  Finding an edge: In the CO2 space, Sanhua is focusing on product development as a way to edge out established competitors. “Our future CO2 ball valves have been designed to integrate a service valve instead of a Schrader valve loading access in order to have an increased passage section that avoids the risk of dry ice formation,” Bisco said.   “Some models of CO2 ball valves will integrate a check valve, while the series for transcritical applications will have a patented design aimed at true bidirectionality,” Bisco added. “These valves will adopt a ball without a hole typically used during pump down to remove the gas trapped in the ball itself. The goal is to simplify installation and reduce the possibility of technical error by installers while maintaining the very high safety standards of the product even in the event of an accidental increase in internal pressure.”  Quotable: “We try to take advantage of the advantage of the newcomer: being able to identify the critical points of existing products and intervene in a targeted way, bringing products to the market that can solve these critical issues,” Bisco said.</t>
+          <t>In an ongoing study of North Carolina firefighters, Duke University researchers are examining a potential link between PFAS exposure and biomarkers of thyroid dysfunction and disease.  This study includes trifluoroacetic acid (TFA), a degradation product of some fluorine-containing gases and other substances, and it is one of the first studies to investigate human health outcomes related to TFA exposure.
+While the researchers found that levels of one thyroid antibody was correlated in a small number of firefighters who had TFA in their blood serum, the results to date are inconclusive.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46002</v>
+        <v>46055</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Components manufacturer Sanhua has announced that it will begin supplying “complete packages” of “coordinated and compatible components” for commercial refrigeration systems using propane (R290) and CO2 (R744) refrigerants. The product packages are part of the company’s 2025–2030 roadmap, which is oriented around natural refrigerants and integrated component packages. Federico Bisco, Technical Director of Sanhua Europe, said the company “has deliberately chosen not to present itself as a manufacturer of finished systems.” Rather, its goal is to help manufacturers reduce the complexity of sourcing components, lower costs through bulk purchases and simplify approving and testing systems. Sanhua is making its product packages available for three types of commercial refrigeration systems: propane plug-ins, propane waterloops and CO2 condensing units. The propane plug-in package: Sanhua said it’s already able to cover “more than 90%” of the components needed for propane plug-in applications.  A product package for propane plug-ins includes filters, solenoid valves, thermostatic expansion valve, electronic expansion valve, exchangers, taps, sensors, electronic controllers, inverters and thermostats. “Package integration allows OEMs to reduce the bill of materials and facilitate system approval,” Sanhua said.  The waterloop package: Sanhua offers three types of product packages for R290 waterloops.  Basic (with mechanical valve), smart (with electronic valve and sensors) and plus (with inverter and digital controller). The product packages are designed for applications where compactness and flexibility are crucial, Sanhua said, and are a fit for small-format grocery stores, convenience stores and retrofits of existing systems.  The CO2 condensing unit package: Sanhua’s product package for CO2 condensing units will include “all critical components,” including pulse expansion valves, smart sensors, heat exchangers, controllers and safety valves. The product package is expected to be available by the end of 2026, and Sanhua is initially targeting CO2 condensing units under 40kW (11.3TR), although it plans to expand the product package to transcritical racks with a capacity of up to 100kW (28.4TR).  “The main challenge is to make CO2 condensing units competitive with HFO solutions,” Bisco said. “Costs remain two to three times higher, but increased volumes and standardized designs are expected to narrow the gap.”  Finding an edge: In the CO2 space, Sanhua is focusing on product development as a way to edge out established competitors. “Our future CO2 ball valves have been designed to integrate a service valve instead of a Schrader valve loading access in order to have an increased passage section that avoids the risk of dry ice formation,” Bisco said.   “Some models of CO2 ball valves will integrate a check valve, while the series for transcritical applications will have a patented design aimed at true bidirectionality,” Bisco added. “These valves will adopt a ball without a hole typically used during pump down to remove the gas trapped in the ball itself. The goal is to simplify installation and reduce the possibility of technical error by installers while maintaining the very high safety standards of the product even in the event of an accidental increase in internal pressure.”  Quotable: “We try to take advantage of the advantage of the newcomer: being able to identify the critical points of existing products and intervene in a targeted way, bringing products to the market that can solve these critical issues,” Bisco said.</t>
+          <t>In an ongoing study of North Carolina firefighters, Duke University researchers are examining a potential link between PFAS exposure and biomarkers of thyroid dysfunction and disease.  This study includes trifluoroacetic acid (TFA), a degradation product of some fluorine-containing gases and other substances, and it is one of the first studies to investigate human health outcomes related to TFA exposure.
+While the researchers found that levels of one thyroid antibody was correlated in a small number of firefighters who had TFA in their blood serum, the results to date are inconclusive.
+The lead researcher in the study is environmental chemist and exposure scientist Heather Stapleton,  a Professor of Environmental Health at Duke University and Director of Duke’s Superfund Research Center. She described the firefighter study at the 46th Annual Meeting of the Society of Environmental Toxicology and Chemistry (SETAC) in Portland, Oregon, held November 16–20, 2025.
+The study is looking broadly at PFAS and its potential association with thyroid disease, Stapleton said. “TFA happens to be one of the PFAS we are including, but this study did not set out to focus on TFA.”
+TFA is regarded by scientists as an ultrashort-chain PFAS (per- and polyfluoroalkyl substance), or “forever chemical”; it has two carbon atoms, one attached to three fluorine atoms. Longer-chain PFAS such as PFOA (perfluorooctanoic acid) and PFOS (perfluorooctanesulfonic acid) are linked to thyroid disease and to kidney and testicular cancer in the case of PFOA, among  other adverse health outcomes.
+TFA also falls under the category of haloacetic acids such as DCA (dichloroacetic acid) and TCA (trichloroacetic acid), which are considered potential human carcinogens and disruptive to thyroid function. As a haloacetic acid, TFA is a substance that “we should look at,” said Stapleton at the SETAC conference.
+The TFA found in the study is not correlated with any of the longer-chain and legacy PFAS, making it easier to assess independently in statistical models. But it is highly correlated with the ultrashort-chain (three-carbon) perfluoropropionic acid (PFPrA), suggesting that TFA and PFPrA may have “unique exposure sources” compared to other PFAS commonly studied in firefighters, it said.
+As a haloacetic acid, TFA is a substance that “we should look at.”
+Heather Stapleton, Professor of Environmental Health at Duke University
+Stapleton acknowledged that there could be a “mixture effect” where TFA would work in concert with other PFAS in impacting thyroid function. “We’re hoping to explore that but we’re trying to get more data before we run those models.”
+TFA itself has been found harmful in low concentrations to lab animals, sounding alarms about its potential effect on humans, especially over long-term exposure as TFA builds up in the environment. The European Chemicals Agency (ECHA) is evaluating  a German proposal to classify TFA as reproductively toxic under the EU’s classification, labelling and packaging (CLP) regulation.
+In defending the use of TFA-producing refrigerants, (notably HFO-1234yf), the fluorochemical Industry points to the UN Environment Programme (UNEP) and its 2022 Environmental Effects Assessment Panel (EEAP) report. The report says that TFA is not bioaccumulative, is “not expected to pose significant risk to humans or the environment at the present time” and “is unlikely to cause adverse effects out to 2100.” The report does not comment on the contribution of pesticides and other precursors to TFA since they don’t fall under the purview of the Montreal Protocol, under which UNEP is an implementing agency.
+Chemours, which operates in North Carolina, told state regulators last year that “based on risk assessment modelling and available toxicological data for similar compounds, [TFA] is not believed to be harmful to human health or the environment.”
+Part of a national study
+Since July 2024, the Duke researchers have been analyzing concentrations of 54 PFAS in the blood serum of more than 700 firefighters (94% male) in North Carolina, part of the National Firefighter Cancer Cohort Study (FFCCS) that was launched in 2018. The researchers are particularly interested in “examining associations between exposure to PFAS such as TFA and the risk for thyroid disease among firefighters,” said Stapleton
+In North Carolina, environmental TFA in the Cape Fear River and drinking water has been linked to emissions from a Chemours facility in Fayetteville as a byproduct of chemicals producer there. But TFA is also generated by the complete atmospheric breakdown in under two weeks of fugitive emissions of the refrigerant HFO-1234yf and the partial breakdown of other fluorinated refrigerants, as well as the decomposition of certain agricultural pesticides and pharmaceuticals, among other sources. HFO-1234yf is widely used in car air-conditioning and in blends with HFC refrigerants used in supermarket and cold-storage refrigeration.
+ Among the PFAS analyzed in the Duke study, TFA was the most abundant compound in blood serum of the first 516 firefighters with a 100% detection frequency, a median concentration of 20.1 ng/g and a maximum concentration of 570 ng/g, according to the abstract. The next most abundant PFAS was PFOS, with a median serum concentration of 3.62 ng/g.
+TFA levels were not associated with participant age, sex or years of firefighting service, in contrast to other legacy PFAS measured, the abstract said.
+Heather Stapleton, Duke University, at the 2025 Society of Environmental Toxicology and Chemistry (SETAC) conference in Portland, Oregon.
+Stapleton noted that TFA levels are “significantly higher” – about 15% – in spring, summer and fall, compared to measurements from participants who were recruited in the winter; she did not offer an explanation for the difference. The Duke team plans to look at the ambient temperature on the days they collected blood samples. Their findings correlate with a 2025 study by Canadian researchers, which found that the amount of TFA in the atmosphere, formed by the oxidation of HFO-1234yf and other f-gases, is greatest in the summer and near urban areas, consistent with the leakage of HFO-1234yf from mobile air conditioners (MAC).
+The TFA levels found in the firefighters exceeds that in blood serum in other studies, including a recent one done at North Carolina State University that reported 17ng/mL and a 2023 study of Indiana households where it was found to be 6ng/mL.
+The researchers at Duke have compared their overall PFAS data with that of the study at North Carolina State University, where researchers have been analyzing blood samples from the general population in Wilmington, North Carolina. “When we make that comparison, our levels are actually pretty similar, with the exception of PFHxS [perfluorohexane sulfonic acid], which is clearly elevated in the firefighters,” said Stapleton in her SETAC presentation.
+Higher cancer rates in firefighters
+The Duke researchers explored potential associations between TFA and thyroid hormones in the study’s firefighter group. Stapleton noted that firefighters reportedly have higher rates of thyroid cancer and higher levels of thyroid autoantibodies than the general population.
+Preliminary findings, the abstract said, “highlight the prominence of TFA as a novel PFAS of concern in firefighters and point to potential associations with thyroid-related biomarkers.” However, Stapleton cautioned at her SETAC presentation that more data is required to come to any conclusions about the effect of TFA on the thyroid.
+“It’s important to remember that most of those measurements are still at a thyroid antibody level that’s considered normal or background,” she said. “it’s not above the threshold for what a medical doctor would refer to as positive or high.”
+The researchers conducted a pilot analysis for the presence of two thyroid autoantibodies – thyroglobulin antibody (TGab) and thyroid peroxidase antibody (TPOab) – in 20 firefighters; these antibodies can attack the thyroid and cause autoimmune dysfunction such as hypothyroidism and Graves’ disease (hyperthyroidism).
+As of November she reported seeing “a number of firefighters testing positive for thyroid antibodies right now – four for TGab and seven for TPOab, which does seem higher than normal for males,” said Stapleton. Most of the samples are restricted to male firefighters, who make up 94% of the study participants.
+In the initial batch of TGab results, the Duke researchers “observed a significant and positive correlation between serum TFA and continuous TGab levels [correlation coefficient r = 0.54], raising questions about a possible immunomodulatory role for TFA,” the abstract said. However, Stapleton said at the SETAC conference, “as more data has come in from other batches, [the TFA–TGab link] has been muted a bit.” Overall, the correlation is 0.18, which is “almost barely statistically significant. So we’ll see if this changes as we collect more data.”
+Stapleton also reported at SETAC having data on levels of free thyroxine (T4) and thyroid stimulating hormone (TSH) – two key hormones involved in metabolic regulation – as well as TFA measurements in 249 firefighters. Her team found “somewhat positive but not statistically significant associations” between TFA and TSH: the higher the TFA, the higher the TSH, but no correlation with T4. These findings were separate from the antibody results, she said; the firefighters that were positive for thyroid antibodies did not have abnormal thyroid hormone levels.
+The Duke team plans to start investigating how much TFA levels in drinking water in North Carolina predict TFA levels in blood serum for the firefighters in the study.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/sanhua-to-offer-complete-packages-of-components-for-co2-and-propane-commercial-refrigeration-systems/</t>
+          <t>https://naturalrefrigerants.com/news/duke-university-researchers-study-potential-link-between-pfas-including-tfa-and-thyroid-dysfunction-in-firefighters/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ATMO Europe: Copeland’s Decentralized CO2 Solution Cuts Auchan Supermarket Retrofit Cost by 6% Compared to Conventional CO2 Rack</t>
+          <t>Part 1: Why Penta Infra Chose Secon’s R290 Chillers for Its New Colocation Facility in Hamburg</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Compared to a conventional CO2 (R744) rack, U.S. components manufacturer Copeland saved French retail group Auchan 6% in capital costs in a supermarket retrofit using a decentralized CO2 solution, according to Fabian Gantois, Manager of Retailer Sales and End Users at the manufacturing company. Gantois, joined by Auchan’s Technical Asset Director Jean-Baptiste Laurencon, outlined the benefits of the modular CO2 outdoor condensing units (OCUs) when used in retrofits and new builds during a presentation at the ATMOsphere (ATMO) Europe Summit 2025. The event, organized by ATMOSphere, publisher of NaturalRefrigerants.com, was held November 24–25 in Padova, Italy. “By eliminating the need for a machine room, CO2 decentralized systems could cut the CAPEX of new stores by up to 10% compared to centralized racks,” Gantois said, adding that the estimate reflects savings of roughly €16,000 ($18,500) per 20m2 (215ft2). “After working with the manufacturer on a successful energy–saving refrigeration deployment in Senegal, we seized the opportunity to be the first to use Copeland’s CO2 decentralized solution in a retrofit of a store in France,” Laurencon said. The installation occurred in June 2024 as part of a pilot test. Retrofit details: The 2,000m2 (21,500ft2) Freyming-Merlebach store previously operated with R448A racks supplying 80kW (22.7TR) of medium-temperature (MT) capacity and R404A systems delivering 20kW (5.7TR) of low-temperature (LT) capacity.  The retrofit installed three CO2 OCUs to meet the MT load and propane (R290) plug-in cabinets for the LT load. Copeland used the R290 units because it was still developing its LT CO2 OCU at the time, Gantois explained. “In 18 months of operation, the new setup maintains the evaporation temperature within 2K [2°C/3.6°F] of the set point, while decreasing the energy consumption of the store by 8%,” Gantois said. It also cuts the store’s carbon emissions by 70 metric tons of CO2e per year compared to the old refrigerants.  MT/LT/heat recovery: Copeland rolled out its full modular CO2 OCU line for commercial applications in May, featuring scroll compressors with vapor injection technology, according to Gantois.  The line covers MT capacities from 15 to 45kW (4.3 to 12.8TR), LT capacities – installed in booster mode with MT units – from 10 to 15kW (2.8 to 4.3TR) and heat recovery for space heating or sanitary water at 40 or 70kW (11.4 or 19.9TR) capacities. The units, with brushless permanent–magnet (BPM) variable speed motors, operate with sound levels of less than 35dB(A) at 10m (32.8ft), making them suitable for urban spaces with noise restrictions. Copeland introduced its first modular CO2 refrigeration unit in 2023 while it was still part of Emerson Climate Technologies. Private investor Blackstone created Copeland as a standalone company in May 2023 when it acquired a majority stake.  Retailer’s next steps: Auchan operates almost 3,000 stores across a total of 12 countries, including locations in Africa and Eastern and Western Europe.  Working within its monetary constraints, the retailer’s strategy is to ultimately switch to CO2 refrigeration, according to Laurencon. The decentralized CO2 scroll units offer a retrofit solution for Auchan’s city stores in Portugal and Spain, its supermarkets and its click-and-collect locations, he added. However, for its hypermarkets, the retailer seeks a hybrid approach using both centralized and decentralized CO2 systems.  Quotable: “With this partnership, we find modularity and scalability,” Laurencon said. “Copeland’s solution is now approved for all of Auchan’s national markets.” “By eliminating the need for a machine room, CO2 decentralized systems could cut the CAPEX of new stores by up to 10% compared to centralized racks.” Fabian Gantois, Manager of Retailer Sales and End Users at Copeland</t>
+          <t>This is an excerpt from an article featured in ATMOsphere’s “Clean Cooling for Data Centers 2025” report, which can be downloaded here. ATMOsphere is the publisher of NaturalRefrigerants.com.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45995</v>
+        <v>46051</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Compared to a conventional CO2 (R744) rack, U.S. components manufacturer Copeland saved French retail group Auchan 6% in capital costs in a supermarket retrofit using a decentralized CO2 solution, according to Fabian Gantois, Manager of Retailer Sales and End Users at the manufacturing company. Gantois, joined by Auchan’s Technical Asset Director Jean-Baptiste Laurencon, outlined the benefits of the modular CO2 outdoor condensing units (OCUs) when used in retrofits and new builds during a presentation at the ATMOsphere (ATMO) Europe Summit 2025. The event, organized by ATMOSphere, publisher of NaturalRefrigerants.com, was held November 24–25 in Padova, Italy. “By eliminating the need for a machine room, CO2 decentralized systems could cut the CAPEX of new stores by up to 10% compared to centralized racks,” Gantois said, adding that the estimate reflects savings of roughly €16,000 ($18,500) per 20m2 (215ft2). “After working with the manufacturer on a successful energy–saving refrigeration deployment in Senegal, we seized the opportunity to be the first to use Copeland’s CO2 decentralized solution in a retrofit of a store in France,” Laurencon said. The installation occurred in June 2024 as part of a pilot test. Retrofit details: The 2,000m2 (21,500ft2) Freyming-Merlebach store previously operated with R448A racks supplying 80kW (22.7TR) of medium-temperature (MT) capacity and R404A systems delivering 20kW (5.7TR) of low-temperature (LT) capacity.  The retrofit installed three CO2 OCUs to meet the MT load and propane (R290) plug-in cabinets for the LT load. Copeland used the R290 units because it was still developing its LT CO2 OCU at the time, Gantois explained. “In 18 months of operation, the new setup maintains the evaporation temperature within 2K [2°C/3.6°F] of the set point, while decreasing the energy consumption of the store by 8%,” Gantois said. It also cuts the store’s carbon emissions by 70 metric tons of CO2e per year compared to the old refrigerants.  MT/LT/heat recovery: Copeland rolled out its full modular CO2 OCU line for commercial applications in May, featuring scroll compressors with vapor injection technology, according to Gantois.  The line covers MT capacities from 15 to 45kW (4.3 to 12.8TR), LT capacities – installed in booster mode with MT units – from 10 to 15kW (2.8 to 4.3TR) and heat recovery for space heating or sanitary water at 40 or 70kW (11.4 or 19.9TR) capacities. The units, with brushless permanent–magnet (BPM) variable speed motors, operate with sound levels of less than 35dB(A) at 10m (32.8ft), making them suitable for urban spaces with noise restrictions. Copeland introduced its first modular CO2 refrigeration unit in 2023 while it was still part of Emerson Climate Technologies. Private investor Blackstone created Copeland as a standalone company in May 2023 when it acquired a majority stake.  Retailer’s next steps: Auchan operates almost 3,000 stores across a total of 12 countries, including locations in Africa and Eastern and Western Europe.  Working within its monetary constraints, the retailer’s strategy is to ultimately switch to CO2 refrigeration, according to Laurencon. The decentralized CO2 scroll units offer a retrofit solution for Auchan’s city stores in Portugal and Spain, its supermarkets and its click-and-collect locations, he added. However, for its hypermarkets, the retailer seeks a hybrid approach using both centralized and decentralized CO2 systems.  Quotable: “With this partnership, we find modularity and scalability,” Laurencon said. “Copeland’s solution is now approved for all of Auchan’s national markets.” “By eliminating the need for a machine room, CO2 decentralized systems could cut the CAPEX of new stores by up to 10% compared to centralized racks.” Fabian Gantois, Manager of Retailer Sales and End Users at Copeland</t>
+          <t>This is an excerpt from an article featured in ATMOsphere’s “Clean Cooling for Data Centers 2025” report, which can be downloaded here. ATMOsphere is the publisher of NaturalRefrigerants.com.
+Secon is a German manufacturer of hydrocarbon heat pumps and chillers founded in 2010 and headquartered in Gondelsheim, Germany. Joachim Schadt, Owner and Managing Director of Secon, said the company works “in the field of critical applications,” such as pharmaceuticals, chemicals, food and infrastructure. The company is particularly active in the DACH region (Germany, Austria and Switzerland). 
+Penta Infra is a provider of edge data centers in Europe. With locations in Germany, France, the Netherlands, Belgium and Denmark, Penta’s solutions range from full-service colocation to build-to-suit data centers. The company was established in 2015 and traditionally worked with synthetic refrigerants but is shifting toward natural refrigerants. A recently built Penta Infra colocation data center in Hamburg is cooled by Secon’s propane (R290) chillers.
+Read: Clean Cooling for Data Centers 2025
+Secon’s hydrocarbon chillers
+Secon manufactures air-cooled and water-cooled chillers and has supplied both for data center projects. Its chillers can contain up to four refrigerant circuits, which reduce the amount of refrigerant that can leak out of an individual circuit. Free cooling is standard, with Schadt noting that it is “the key to achieve low PUE [power usage effectiveness] values.”
+Schadt said Secon’s hydrocarbon chillers are “not designed for the lowest possible price.” Instead, they’re “built for efficiency and operational reliability, which then translates into the lowest possible lifecycle costs,” he said, adding that Secon customizes its chillers for data center projects. 
+“We’re not selling out of a catalog,” Schadt said. “We talk to the customers, their consultants or both to get a feeling for their requirements. In the end, the only ‘identical’ chillers we produce are ones used for the same project.”
+Customization is particularly evident in hydraulics and controls optimization. Secon’s chillers are equipped with ultrasonic flow meters that detect the “real flow” of water in cubic meters per hour as opposed to switches that detect whether water is flowing. The control systems for the chillers also come standard with uninterruptible power supplies (UPS) and automatic transfer switches that move the power supply from one electricity supply to another while the UPS continuously supplies power to the control system in the event of an interruption. 
+“The data center providers always ask, ‘What are your references?’ When you show them references in pharmaceutical applications as well as food and beverage, they trust you.”
+Joachim Schadt,
+Owner and Managing Director of Secon
+Moving to natural refrigerants
+Harmen Laan, Head of Engineering at Penta Infra, said that the transition to hydrocarbon chillers has been challenging, largely because the technology is still considered non-standard within the data center industry. He noted that much of the hesitation stems from unfamiliarity with hydrocarbon-based systems and “persistent myths” that range from concerns about safety and inefficiency to perceptions of outdated technology and the absence of recognized certifications like Eurovent.
+“While these concerns are mostly unfounded, it is true that hydrocarbon chillers generally require a larger physical footprint, which remains a valid consideration,” Laan said.
+To address these concerns, Laan and his team conducted a thorough investigation, benchmarking hydrocarbon solutions against synthetic refrigerant alternatives. This included multiple site visits to Secon’s manufacturing facilities in Croatia and Italy to ensure the systems met the high standards required for “mission-critical operations.”
+Carving out a niche
+Since 2018, Secon has completed 34 data center projects with a total of 95 chillers delivered. The vast majority of those projects have been in Germany. The company currently has 30 projects in the design and tendering phases and is seeing “increased demand in this area,” according to Schadt. The majority of projects are for the DACH region, and the company’s work in “critical fields” helped it enter the space.
+“The data center providers always ask, ‘What are your references?’” Schadt said. “It can’t be a large data center as you are one of the first to approach us about this, but when you show them references in pharmaceutical applications as well as food and beverage, they trust you.”
+He said that the European Union’s F-gas Regulation has driven increased demand for Secon’s hydrocarbon chillers, with the “PFAS issue” also contributing. Schadt said Secon’s data center business has grown by 10% in the past two to three years, and he expects even greater growth in the future.
+In addition to the DACH region, the company has worked on data centers in France, the Netherlands and Denmark. The largest data center Secon has worked on to date – in terms of installed IT power capacity – is 4.4MW. Data center projects in its pipeline range from 1MW to 20MW of installed IT power capacity, with Secon’s chillers providing the entire IT cooling load.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-copelands-decentralized-co2-solution-cuts-auchan-supermarket-retrofit-cost-by-6-compared-to-conventional-co2-rack/</t>
+          <t>https://naturalrefrigerants.com/news/part-1-why-penta-infra-chose-secons-r290-chillers-for-its-new-colocation-facility-in-hamburg/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Agritechnica 2025: Konvekta Showcases CO2-Qube Thermal Management System for Electric Heavy Equipment</t>
+          <t>NASRC Training Event to Address CO2 Knowledge Gap in New York</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>German manufacturer Konvekta showcased CO2-Qube, its CO2 (R744)-based thermal management system for electric heavy equipment, including agriculture and construction vehicles, at Agritechnica 2025. CO2-Qube incorporates the company’s CO2 heat pump technology in electric buses and rail vehicles, with prototypes undergoing performance testing, according to Konvekta. It expects the final product to offer 8kW (2.3TR) of cooling capacity and 8.5kW (2.4TR) of heating. “In response to growing environmental awareness and the resulting regulatory changes – particularly the ban on per– and polyfluoroalkyl substances (PFAS) and other chemical refrigerants – ‘CO2–Qube’ comes into focus as a forward–looking study in the field of air conditioning and heating for electrically powered mobile work machines,” Konvekta said. Agritechnica 2025, considered the world’s largest trade fair for agricultural technology, was held November 9–15 in Hanover, Germany. It featured 2,849 exhibitors from 52 countries and attracted 476,000 visitors from 171 countries. The setup: The system manages the entire thermal load of electric work machines by extracting energy from both ambient air and system components, including the drive train and the battery.  The system, available in 400 or 600V AC with 24V DC, preheats and cools the battery, cools the power electronics and provides heating and cooling for the cabin. Konvekta envisions two final design options: a compact version optimizing service for minimized downtime and a modular one for maximum flexibility. With plug-and-play installation, the heat pump system mounts on the rooftop or the chassis, according to the manufacturer.  The backbone: CO2-Qube operates with an electric AC compressor newly developed by German automotive component specialist Thyssenkrupp Automotive.  “The e–AC Compressor delivers energy efficiency and reliability even under demanding off–road conditions,” Thyssenkrupp said. “By driving innovation in thermal management, [we] contribute to more sustainable mobility solutions – helping agricultural machinery become cleaner, smarter, and more efficient for the challenges ahead.”  Previous accolades: Konvekta won Busworld Europe 2023’s Innovation award for its CO2 heat pump thermal management system for electric double-decker buses.  The system delivers both air-conditioning and heating while consuming only a fraction of the energy required by traditional MAC systems or electric heaters, which Konvekta called “a milestone in the development of sustainable technologies in the public transport sector.” In 2023 the Konvekta improved its CO2 heat pump technology for e-buses with a “refrigerant charge balancing” system that it said improves the range by increasing the efficiency of heating and cooling.  Quotable: “CO2–Qube impresses with its PFAS–free CO2 heat pump technology,” Konvekta said. “[It] shows what sustainable thermal management in agricultural and commercial vehicles can look like.” “[CO2–Qube] shows what sustainable thermal management in agricultural and commercial vehicles can look like.” Konvekta</t>
+          <t>The North American Sustainable Refrigeration Council (NASRC) will be holding its next free training event for commercial and industrial refrigeration technicians in Poughkeepsie, New York, February 10–12, addressing a perceived knowledge gap among New York State technicians regarding CO2 (R744) refrigeration.
+It will be NASRC’s 12th technician training event since launching them in April 2023 in Irwindale, California, and the first to be held in New York State. The Poughkeepsie event, which will take place at the DoubleTree by Hilton, will focus on CO2 refrigeration, with some coverage of propane (R290) systems.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45993</v>
+        <v>46049</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>German manufacturer Konvekta showcased CO2-Qube, its CO2 (R744)-based thermal management system for electric heavy equipment, including agriculture and construction vehicles, at Agritechnica 2025. CO2-Qube incorporates the company’s CO2 heat pump technology in electric buses and rail vehicles, with prototypes undergoing performance testing, according to Konvekta. It expects the final product to offer 8kW (2.3TR) of cooling capacity and 8.5kW (2.4TR) of heating. “In response to growing environmental awareness and the resulting regulatory changes – particularly the ban on per– and polyfluoroalkyl substances (PFAS) and other chemical refrigerants – ‘CO2–Qube’ comes into focus as a forward–looking study in the field of air conditioning and heating for electrically powered mobile work machines,” Konvekta said. Agritechnica 2025, considered the world’s largest trade fair for agricultural technology, was held November 9–15 in Hanover, Germany. It featured 2,849 exhibitors from 52 countries and attracted 476,000 visitors from 171 countries. The setup: The system manages the entire thermal load of electric work machines by extracting energy from both ambient air and system components, including the drive train and the battery.  The system, available in 400 or 600V AC with 24V DC, preheats and cools the battery, cools the power electronics and provides heating and cooling for the cabin. Konvekta envisions two final design options: a compact version optimizing service for minimized downtime and a modular one for maximum flexibility. With plug-and-play installation, the heat pump system mounts on the rooftop or the chassis, according to the manufacturer.  The backbone: CO2-Qube operates with an electric AC compressor newly developed by German automotive component specialist Thyssenkrupp Automotive.  “The e–AC Compressor delivers energy efficiency and reliability even under demanding off–road conditions,” Thyssenkrupp said. “By driving innovation in thermal management, [we] contribute to more sustainable mobility solutions – helping agricultural machinery become cleaner, smarter, and more efficient for the challenges ahead.”  Previous accolades: Konvekta won Busworld Europe 2023’s Innovation award for its CO2 heat pump thermal management system for electric double-decker buses.  The system delivers both air-conditioning and heating while consuming only a fraction of the energy required by traditional MAC systems or electric heaters, which Konvekta called “a milestone in the development of sustainable technologies in the public transport sector.” In 2023 the Konvekta improved its CO2 heat pump technology for e-buses with a “refrigerant charge balancing” system that it said improves the range by increasing the efficiency of heating and cooling.  Quotable: “CO2–Qube impresses with its PFAS–free CO2 heat pump technology,” Konvekta said. “[It] shows what sustainable thermal management in agricultural and commercial vehicles can look like.” “[CO2–Qube] shows what sustainable thermal management in agricultural and commercial vehicles can look like.” Konvekta</t>
+          <t>The North American Sustainable Refrigeration Council (NASRC) will be holding its next free training event for commercial and industrial refrigeration technicians in Poughkeepsie, New York, February 10–12, addressing a perceived knowledge gap among New York State technicians regarding CO2 (R744) refrigeration.
+It will be NASRC’s 12th technician training event since launching them in April 2023 in Irwindale, California, and the first to be held in New York State. The Poughkeepsie event, which will take place at the DoubleTree by Hilton, will focus on CO2 refrigeration, with some coverage of propane (R290) systems. It will be  co-hosted by New Yorkers for Clean Power and the Cornell Cooperative Extension Smart Energy Choices – Mid-Hudson.
+“What’s surprising about New York is that there’s a lot of CO2 systems but there are very few technicians who have actually worked on CO2,” said Danielle Wright, Executive Director of the NASRC, a nonprofit that aims to overcome obstacles to the adoption of natural refrigerants. “So we’re really focused on covering the basics and getting them that foundation.” New York State, which has some of the most aggressive HFC regulations in the U.S., recently withstood a legal challenge to those regulations.
+The event will offer classroom and some hands-on sessions as well as an exhibit hall featuring natural refrigerant products and services. Topics include everything from CO2 oil management and compressor troubleshooting to adiabatic cooling and rack start-up.
+Trainers will come from the following organizations: Hillphoenix, Copeland, Energy Recovery, Bitzer, Parker Hannifin/Sporlan, Carel, Kysor Warren, BAC, FLō, Dorin, Mueller Streamline, Zero Zone; Future Green Now, NASRC and the New York Department of Environmental Conservation. Copeland plans to bring its mobile CO2 unit while Baltimore Aircoil (BAC) will showcase its Trillium condenser. In addition, Bitzer and Dorin will demonstrate compressor tear-down.
+“What’s surprising about New York is that there’s a lot of CO2 systems but there are very few technicians who have actually worked on CO2.”
+Danielle Wright, Executive Director of the NASRC
+The final day, February 12, will feature a morning workshop with NASRC Trainer Rusty Walker on remodeling  with CO2 booster systems. This course will provide practical methods for converting an operating store from an HFC rack system to a CO2 system with minimal disruption.
+In addition, on February 11 HVAC&amp;R trade school students and faculty can attend a free career fair with employers from the refrigeration industry. Participants will learn about career opportunities, connect with industry employers and gain exposure to the latest refrigeration technologies. “These students often get pushed towards the HVAC side, so we’re trying to get them more focused and tuned into the refrigeration side and give them an introduction to what a career in refrigeration would be like,” said Wright.
+R-TRADE program
+In 2024 the NASRC formalized its training program with the launch of R-TRADE (refrigeration technician recruitment, advancement, development and education) with seed funding from five major stakeholders in the U.S. grocery retail sector: Albertsons, Amazon, Costco, Kroger and Walmart. The NASRC describes R-TRADE as a nationwide workforce development program with the goal of training more than 14,000 refrigeration technicians.  Last year the nonprofit added the R-TRADE Supporters program, which enables organizations to contribute funding directly to the training initiative without becoming a member of the NASRC.
+The NASRC will be hosting its next training events in St. Louis and San Antonio in March and Irwindale in April. Wright noted that the St Louis event will offer the first industrial track and in Irwindale, NASRC will offer a CO2-remote-condensing-unit showcase. The latter event will be geared “just as much towards end users as technicians because we want the end users to come in see these new products and get interested in using them,” she said.
+“Every event evolves as we learn something new,” said Wright.  “For instance, the very first event didn’t have any hands-on component and now we’re incorporating that more and more. We always tinker with the format and the length of the presentations, trying to balance getting as many sessions in as possible with making sure that technicians can actually attend all the sessions that they want to attend.”
+The NASRC’s training program aims to overcome a perennial challenge in the natural refrigerants industry – developing enough technicians knowledgeable in natural refrigerant technologies. A confident, well-trained technician workforce “is the foundation for a successful transition” to natural refrigerants, wrote Morgan Vanzo, Senior Director of the NASRC, in an expert opinion piece last year.
+ “When technicians have the expertise to install, maintain and service the full range of natural refrigerant systems, the industry gains the capacity to move forward quickly and effectively,” added Vanzo. “These skills drive measurable benefits, like enhanced system performance, improved service reliability and reduced operational costs, while securing compliance and positioning businesses for long-term success.”
+ATMOsphere, publisher of NaturalRefrigerants.com, will be holding its 2026 ATMOsphere America conference on natural refrigerants in Tarrytown, N.Y., just north of New York City, June 2–3.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/agritechnica-2025-konvekta-showcases-co2-qube-thermal-management-system-for-electric-heavy-equipment/</t>
+          <t>https://naturalrefrigerants.com/news/nasrc-training-event-to-address-co2-knowledge-gap-in-new-york/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Copeland Takes Step Toward Public Listing With Confidential U.S. IPO Filing</t>
+          <t>Canadian Researchers Find Marked Decline of Atmospheric TFA During COVID</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>U.S. component manufacturer Copeland, backed by the private equity firm Blackstone, has taken its first step toward public listing with the confidential filing of a proposed initial public offering with the U.S. Securities and Exchange Commission (SEC). Previously, Copeland operated as a division of the global industrial technology and engineering giant Emerson. Blackstone’s 2023 acquisition of a 60% majority stake in Emerson’s Climate Technologies division led to the creation of the standalone company, valued at $14 billion (€13 billion). Emerson sold its remaining 40% stake in Copeland to Blackstone in June 2024. “Since becoming a standalone company, we’ve increased our investments in R&amp;D,” said Copeland CEO Ross Shuster. “We’ve launched over 120 new products to the marketplace and filed for 430 new patents.” “Taking a long–term view, we’ve helped Copeland lower costs, grow its manufacturing footprint, optimize pricing and enhance employee engagement,” said Seth Meisel, Senior Managing Director at Blackstone. “A shared ownership program provides broad-based employee eligibility for equity-linked bonuses.” Copeland produces products for commercial and industrial applications, including CO2 (R744) compressors and controls, small-scale propane (R290) compressors and industrial-sized Vilter-brand ammonia (R717) compressors. In fiscal year 2024, the company generated $4.75 billion (€4.12 billion) in revenue, according to Copeland’s 2025 Global Impact Report. What’s next: With its IPO filing, Copeland plans to offer Class A common stock on a U.S. exchange.   The number of shares and the price per share, although not yet determined, will be subject to the market and SEC review. As part of the filing, Copeland detailed the company’s business description, ownership structure, financial statements, expected use of IPO proceeds, risk factors and a preliminary share price. Copeland’s formal IPO underwriter mandates could start in 2026, according to Bloomberg News, with Blackstone engaging several banks, including Morgan Stanley, Barclays, Goldman Sachs and Jefferies.  Recent accolade: Copeland’s transcritical CO2 scroll compressor with dynamic vapor injection technology won the 2026 AHR Expo (International Air-Conditioning, Heating, Refrigerating Exposition) Innovation Award in the refrigeration category. The event will take place February 2–4, 2026, in Las Vegas.  The compressor, designed for medium-temperature, distributed CO2 refrigeration, supports small-supermarket and convenience-store applications. Its ZTI model offers cooling capacities from 7.7 to 18.6kW (2.2 to 5.3TR).  Various markets: Copeland’s products cover numerous thermal applications.  Vehicle HVAC manufacturer Aurora Netherlands uses Copeland’s R290 scroll compressor in its dual secondary loop propane heat pump HVAC system for electric buses. In October Copeland announced plans to acquire Sustainable Process Heat, a German company specializing in industrial-sized hydrocarbon high-temperature heat pumps. Under its Vitler brand, the manufacturer supplied a 1.5MW (426.5TR) water-to-water ammonia heat pump to a Canadian dairy processing facility.  Quotable: “It’s different when everybody has skin in the game,” said Paul Lundstrom, Copeland’s CFO. “With the shared ownership program, people throughout the company are identifying things that we should think differently about to harness the energy in the system.” “Since becoming a standalone company, we’ve launched over 120 new products to the marketplace and filed for 430 new patents.” Ross Shuster, CEO Copeland</t>
+          <t>Researchers at York University in Toronto, Canada, have found that the amount of trifluoroacetic acid (TFA) in the atmospheric declined during the COVID-19 pandemic in 2020 by a factor of 2–5, suggesting that sources of TFA in Toronto are mainly short-lived HFO precursors like HFO-123ryf.
+The findings are described in a study – “Atmospheric Removal of Trifluoroacetic Acid by Dry and Wet Deposition: A Multiyear Analysis in Toronto” –  published January 29 in the journal Environmental Science &amp; Technology Letters.
+TFA is regarded by scientists as an ultrashort-chain PFAS (per- and polyfluoroalkyl substance), or “forever chemical” that persists in the environment; it has two carbon atoms, one attached to three fluorine atoms.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45989</v>
+        <v>46056</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>U.S. component manufacturer Copeland, backed by the private equity firm Blackstone, has taken its first step toward public listing with the confidential filing of a proposed initial public offering with the U.S. Securities and Exchange Commission (SEC). Previously, Copeland operated as a division of the global industrial technology and engineering giant Emerson. Blackstone’s 2023 acquisition of a 60% majority stake in Emerson’s Climate Technologies division led to the creation of the standalone company, valued at $14 billion (€13 billion). Emerson sold its remaining 40% stake in Copeland to Blackstone in June 2024. “Since becoming a standalone company, we’ve increased our investments in R&amp;D,” said Copeland CEO Ross Shuster. “We’ve launched over 120 new products to the marketplace and filed for 430 new patents.” “Taking a long–term view, we’ve helped Copeland lower costs, grow its manufacturing footprint, optimize pricing and enhance employee engagement,” said Seth Meisel, Senior Managing Director at Blackstone. “A shared ownership program provides broad-based employee eligibility for equity-linked bonuses.” Copeland produces products for commercial and industrial applications, including CO2 (R744) compressors and controls, small-scale propane (R290) compressors and industrial-sized Vilter-brand ammonia (R717) compressors. In fiscal year 2024, the company generated $4.75 billion (€4.12 billion) in revenue, according to Copeland’s 2025 Global Impact Report. What’s next: With its IPO filing, Copeland plans to offer Class A common stock on a U.S. exchange.   The number of shares and the price per share, although not yet determined, will be subject to the market and SEC review. As part of the filing, Copeland detailed the company’s business description, ownership structure, financial statements, expected use of IPO proceeds, risk factors and a preliminary share price. Copeland’s formal IPO underwriter mandates could start in 2026, according to Bloomberg News, with Blackstone engaging several banks, including Morgan Stanley, Barclays, Goldman Sachs and Jefferies.  Recent accolade: Copeland’s transcritical CO2 scroll compressor with dynamic vapor injection technology won the 2026 AHR Expo (International Air-Conditioning, Heating, Refrigerating Exposition) Innovation Award in the refrigeration category. The event will take place February 2–4, 2026, in Las Vegas.  The compressor, designed for medium-temperature, distributed CO2 refrigeration, supports small-supermarket and convenience-store applications. Its ZTI model offers cooling capacities from 7.7 to 18.6kW (2.2 to 5.3TR).  Various markets: Copeland’s products cover numerous thermal applications.  Vehicle HVAC manufacturer Aurora Netherlands uses Copeland’s R290 scroll compressor in its dual secondary loop propane heat pump HVAC system for electric buses. In October Copeland announced plans to acquire Sustainable Process Heat, a German company specializing in industrial-sized hydrocarbon high-temperature heat pumps. Under its Vitler brand, the manufacturer supplied a 1.5MW (426.5TR) water-to-water ammonia heat pump to a Canadian dairy processing facility.  Quotable: “It’s different when everybody has skin in the game,” said Paul Lundstrom, Copeland’s CFO. “With the shared ownership program, people throughout the company are identifying things that we should think differently about to harness the energy in the system.” “Since becoming a standalone company, we’ve launched over 120 new products to the marketplace and filed for 430 new patents.” Ross Shuster, CEO Copeland</t>
+          <t>Researchers at York University in Toronto, Canada, have found that the amount of trifluoroacetic acid (TFA) in the atmospheric declined during the COVID-19 pandemic in 2020 by a factor of 2–5, suggesting that sources of TFA in Toronto are mainly short-lived HFO precursors like HFO-123ryf.
+The findings are described in a study – “Atmospheric Removal of Trifluoroacetic Acid by Dry and Wet Deposition: A Multiyear Analysis in Toronto” –  published January 29 in the journal Environmental Science &amp; Technology Letters.
+TFA is regarded by scientists as an ultrashort-chain PFAS (per- and polyfluoroalkyl substance), or “forever chemical” that persists in the environment; it has two carbon atoms, one attached to three fluorine atoms. Longer-chain PFAS such as PFOA (perfluorooctanoic acid) and PFOS (perfluorooctanesulfonic acid) are linked to thyroid disease and to kidney and testicular cancer in the case of PFOA, among  other adverse health outcomes.
+While atmospheric deposition is regarded as a major source of TFA, it also generated as a degradation byproduct of certain pesticides, pharmaceuticals and other PFAS, as well as from industrial releases and sewage treatment.
+The study took monthly measurements between 2018 and 2024 of TFA deposition from the atmosphere at an air-quality research station on the roof of York University’s Petrie Science and Engineering Building. The researchers linked the marked decline of TFA during the pandemic of 2020 to the reduction in usage of HFO-1234yf as a refrigerant, notably in car air-conditioning.
+“When we turned off the tap, so to speak, and we all went home and stopped normal activities, we saw a really quick response, a dramatic reduction of TFA,” said Cora Young, a Professor and Atmospheric Chemist at York University and senior author of the study, in a press release.
+HFO-1234yf that leaks from cars into the atmosphere converts entirely via photo-oxidation into TFA within about 12 days. In car air-conditioning HFO-1234yf, with a GWP of less than one, has largely replaced HFC-134a, which has a 100-year GWP of 1,530 and an atmospheric lifetime of 14 years, breaking down into TFA at a rate of 7–20%.
+“I was so surprised when we saw that it had decreased during the pandemic, but I had to double- and triple-check the data because I didn’t believe it at first.”
+Cora Young, Professor and Atmospheric Chemist at York University
+TFA formed in the atmosphere is largely absorbed in rain or snow and deposited into the environment but some comes down as “dry” deposition, such as when gaseous TFA land on surfaces and forms a layer of dust. A 2025 study by North Carolina State and Duke University researchers found TFA in 89% of household dust samples linked to PFAS emissions from a fluorochemical plant.
+Young said the “real surprise” in the study is that it points to TFA being formed from short-lived chemical precursors – primarily HFO-1234yf – emitted into the atmosphere. “I was so surprised when we saw that it had decreased during the pandemic, but I had to double- and triple-check the data because I didn’t believe it at first.”
+She also noted in an email communication that it has been difficult previously to distinguish between TFA coming from the longer-lived HFC precursors and the short-lived HFO precursors. “I think this is compelling evidence that short-lived are already significant contributors.”
+Peaking in the summer
+As the COVID pandemic subsided and normal activities resumed, TFA levels in the atmosphere crept back up, the researchers found. The peak levels occur in the summer when there is more light, which triggers the transformation of f-gases into TFA. Last year, Young was part of a study that found the amount of TFA in the atmosphere is greatest in the summer and near urban areas, consistent with the leakage of HFO-1234yf from mobile air conditioners. Her group also determined in a 2024 study that the TFA in the atmosphere in Toronto was coming from atmospheric formation.
+The new study looked at the relative contributions of wet, dry and total deposition of TFA from the atmosphere between 2018 and 2024. According to the study abstract, the researchers collected 103 total samples and 98 wet samples with TFA concentrations ranging from 0.07–4.55mcg/L and 0.09–3.19mcg/L, respectively. The median dry deposition flux (106mcg/m2 per year ) accounted for 0–94% (median 37%) of the total TFA deposition, higher and more variable than model estimates, the abstract said. “These results provide the first field-based quantification of TFA in dry deposition, demonstrating that it is a significant and previously underrepresented removal pathway,” it added.
+Young saw a silver lining in the new study’s findings: “I see this as very important for framing regulation of these chemicals,” she said. “If short-lived precursors are already a dominant source, then regulation would be very effective.”
+Some regions of the world are looking at regulating the emissions of HFO-1234yf and other HFOs that generate TFA, notably Canada, some U.S. states and especially the EU. On the other hand, the U.S. Environmental Protection Agency (EPA) last year approved pesticides known to break down into TFA.
+ Potential health effects
+Young acknowledged that the health effects of long-term exposure to TFA on people and wildlife are still unknown. However, she added, its concentrations in the environment are “orders of magnitude” higher than that of bioaccumulative, cancer-linked PFAS like PFOA.
+While TFA is not thought to bioaccumulate in humans, it’s “been found to accumulate in plants and can be found in the food people and wildlife eat. It has even been found in human blood,” said Young. “Our exposure could still be quite high, even if it’s not bioaccumulating.”
+Research around the world is beginning to shed light on the potential toxicity of TFA. TFA has been found harmful in low concentrations to lab animals, sounding alarms about its potential effect on humans, especially over long-term exposure as TFA builds up in the environment. The European Chemicals Agency (ECHA) is evaluating  a German proposal to classify TFA as reproductively toxic under the EU’s classification, labelling and packaging (CLP) regulation.
+The rooftop air-quality research station at York University used to measure atmospheric TFA deposition. Image from York University
+In the U.S., Duke University researchers are examining a potential link between firefighters’ exposure to PFAS, including TFA, and biomarkers of thyroid dysfunction and disease – one of the first studies to investigate human health outcomes related to TFA exposure. This study has found TFA in human blood serum, as have studies by North Carolina State University and Emory University.
+In defending the use of TFA-producing refrigerants, (notably HFO-1234yf), the fluorochemical Industry points to the UN Environment Programme (UNEP) and its 2022 Environmental Effects Assessment Panel (EEAP) report. The report says that TFA is not bioaccumulative, is “not expected to pose significant risk to humans or the environment at the present time” and “is unlikely to cause adverse effects out to 2100.” The report does not comment on the contribution of pesticides and other precursors to TFA since they don’t fall under the purview of the Montreal Protocol, under which UNEP is an implementing agency.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/copeland-takes-step-toward-public-listing-with-confidential-u-s-ipo-filing/</t>
+          <t>https://naturalrefrigerants.com/news/canadian-researchers-find-marked-decline-of-atmospheric-tfa-during-covid/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ATMO Europe: Taking a Stand on PFAS</t>
+          <t>Haier Carrier CO2 Heat Pump Provides Comfort Heating and Cooling for New AstraZeneca Pharmaceutical Park in China</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>In 2014, Malene Teller Blume, Quality and Development Manager for the Nordic food retailer Coop Trading and its subsidiary Coop Denmark, found herself talking about the chemical pollutant PFAS (per-and polyfluoroalkyl substances) on television as a guest on a popular Danish consumer program. By 2014, PFOA, a type of PFAS, was recognized as a possible carcinogen, and leading experts stated that the TDI (tolerable daily intake) level for PFAS was 100 to 1,000 times too high, with children particularly vulnerable. Teller Blume knew that PFAS was used in packaging for Coop Trading’s more than 4,000 private label products. Without checking with her company, Teller Blume, who is responsible for chemical strategy, decided to say publicly on the program that Coop Trading and Coop Denmark were banning PFAS in its packaging. “[I] couldn’t just say we will look into it, or we will do some monitoring; we need to be very strict about this,” said Teller Blume. “So I decided to say we have a ban. And then the hard work started.” Her manager “trusted my judgment because this was the right thing to do.” After relating this story during a PFAS panel discussion on November 24 at the ATMOsphere (ATMO) Europe Summit 2025 in Padova, Italy, Teller Blume received one of several ovations from attendees. Later that day she accepted, on behalf of Coop Denmark, the ATMO Europe 2025 Best-in-Sector/Retail End User award in recognition of the company’s pioneering work on the PFAS issue and its environmental initiatives. The conference was organized by ATMOsphere, publisher of NaturalRefrigerants.com. “I’ve been dedicated to [eliminating] PFAS since 2014 and besides raising my three children, this is the thing that I’m most proud of,” said Teller Blume. Coop Denmark, at 150 years old the country’s largest retailer with more than 1,000 stores, has also been a leader in the phaseout of HFCs and is installing PFAS-free natural refrigerant systems. A complete phaseout of HFC gases with high global warming potential is planned in accordance with EU regulations, and HFCs have been reduced by 76% since 2018, said Teller Blume. Coop also plans “a technological shift to natural refrigerants” with SBTi (Science-Based Targets initiative)-validated targets. Overall, Coop Denmark aims to reduce CO₂e emissions by 75% in 2025 and 91% by 2030, compared to 2018 levels. Coop Denmark began installing transcritical CO2 systems at its Fakta stores around 2010. (Many Fakta stores were converted to the Coop 365discount format in 2022.)  The retailer has also invested in solar panels, heat pumps, heat recovery and LED lighting, purchased 23 electric delivery vans and installed charging stations at 500 stores, more than half of its locations. First for microwave popcorn By mid-2015 Coop Denmark had banned all PFAS-based paper and cardboard packaging with direct food contact except for microwave popcorn bags, for which there were no PFAS-free alternatives. As an interim step, the retailer pulled microwaveable popcorn from store shelves, but later that year It introduced its own PFAS-free microwaveable popcorn. In seeking a PFAS-free microwave popcorn bag, Coop Denmark worked with its supplier, which discovered that “if they treated the paper with more heat, more water and more mechanical treatment, they didn’t have to use PFAS to cover the inside,” she said. This resulted in the world’s first PFAS-free microwave popcorn bag, making Teller Blume “famous for some months.” The U.S. state of Washington subsequently banned PFAS in food packaging, using the Coop Denmark’s popcorn bag as an inspiration. In 2016 Coop Denmark banned PFAS in outwear, textiles and home textiles. Two years later it prohibited PFAS in cleaning, cosmetics and personal care products, and in 2023 it took aim at PFAS outdoor textiles and garden furniture. In 2024 PFAS frying pans were banned. “I’ve been dedicated to [eliminating] PFAS since 2014 and besides raising my three children, this is the thing that I’m most proud of.” Malene Teller Blume, Coop Denmark Along with product bans, Coop Denmark has also contributed to national anti-PFAS legislation. It started a campaign in 2017 to ban the use of PFAS in paper and cardboard food contact materials (FCM). In September 2019 Denmark announced it would ban PFAS in FCM – the ban went into effect in July 2020 – making it the first country to do so. In addition, Coop Denmark works with organizations like ChemSec to advocate for PFAS bans at the EU level. Teller Blume shared a video explaining how Coop Denmark was able to persuade the Danish parliament to ban PFAS in food packaging. Early on, the company organized a social media campaign, backed by consumers and directed at members of parliament, sparking a debate on the problem of hazardous chemicals. Then, “together with experts, we prepared a complete post for a bill against hazardous chemicals, which could immediately be submitted into parliament,” the video said. “The campaign quickly gained the politicians attention; to ensure that no one missed this important message, we also surrounded the parliament building.” PFAS is not the only chemical contaminant that Coop Denmark has addressed over the course of its history, said Teller Blume; all told the company has taken 185 actions, including bans of PVC (polyvinyl chloride) in packaging in 1991, allergenic preservatives and fragrances in 1995 and bisphenol A in 2016. “We have tried to use early warnings, and also use the precautionary principle to set up requirements,” she said. “If there was a possible further solution, then we have put it in our trade agreements.” Teller Blume has met with leading anti-PFAS figures and environmental activists such as attorney Robert Bilott and scientist Arlene Blum. Years after he first met her, Bilott mentioned to Teller Blume that he has “told your story many times when people are saying that it’s not possible to face up to PFAS.”</t>
+          <t>A newly opened AstraZeneca pharmaceutical park in Qingdao, China, is equipped with a Haier Carrier CO2 (R744) heat pump system that provides comfort heating and cooling across the 54,000m2 (581,251ft2) complex.
+Haier Carrier shared the news in a press release detailing the project as well as a video posted to LinkedIn. The Qingdao site features both offices and R&amp;D facilities.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45988</v>
+        <v>46045</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>In 2014, Malene Teller Blume, Quality and Development Manager for the Nordic food retailer Coop Trading and its subsidiary Coop Denmark, found herself talking about the chemical pollutant PFAS (per-and polyfluoroalkyl substances) on television as a guest on a popular Danish consumer program. By 2014, PFOA, a type of PFAS, was recognized as a possible carcinogen, and leading experts stated that the TDI (tolerable daily intake) level for PFAS was 100 to 1,000 times too high, with children particularly vulnerable. Teller Blume knew that PFAS was used in packaging for Coop Trading’s more than 4,000 private label products. Without checking with her company, Teller Blume, who is responsible for chemical strategy, decided to say publicly on the program that Coop Trading and Coop Denmark were banning PFAS in its packaging. “[I] couldn’t just say we will look into it, or we will do some monitoring; we need to be very strict about this,” said Teller Blume. “So I decided to say we have a ban. And then the hard work started.” Her manager “trusted my judgment because this was the right thing to do.” After relating this story during a PFAS panel discussion on November 24 at the ATMOsphere (ATMO) Europe Summit 2025 in Padova, Italy, Teller Blume received one of several ovations from attendees. Later that day she accepted, on behalf of Coop Denmark, the ATMO Europe 2025 Best-in-Sector/Retail End User award in recognition of the company’s pioneering work on the PFAS issue and its environmental initiatives. The conference was organized by ATMOsphere, publisher of NaturalRefrigerants.com. “I’ve been dedicated to [eliminating] PFAS since 2014 and besides raising my three children, this is the thing that I’m most proud of,” said Teller Blume. Coop Denmark, at 150 years old the country’s largest retailer with more than 1,000 stores, has also been a leader in the phaseout of HFCs and is installing PFAS-free natural refrigerant systems. A complete phaseout of HFC gases with high global warming potential is planned in accordance with EU regulations, and HFCs have been reduced by 76% since 2018, said Teller Blume. Coop also plans “a technological shift to natural refrigerants” with SBTi (Science-Based Targets initiative)-validated targets. Overall, Coop Denmark aims to reduce CO₂e emissions by 75% in 2025 and 91% by 2030, compared to 2018 levels. Coop Denmark began installing transcritical CO2 systems at its Fakta stores around 2010. (Many Fakta stores were converted to the Coop 365discount format in 2022.)  The retailer has also invested in solar panels, heat pumps, heat recovery and LED lighting, purchased 23 electric delivery vans and installed charging stations at 500 stores, more than half of its locations. First for microwave popcorn By mid-2015 Coop Denmark had banned all PFAS-based paper and cardboard packaging with direct food contact except for microwave popcorn bags, for which there were no PFAS-free alternatives. As an interim step, the retailer pulled microwaveable popcorn from store shelves, but later that year It introduced its own PFAS-free microwaveable popcorn. In seeking a PFAS-free microwave popcorn bag, Coop Denmark worked with its supplier, which discovered that “if they treated the paper with more heat, more water and more mechanical treatment, they didn’t have to use PFAS to cover the inside,” she said. This resulted in the world’s first PFAS-free microwave popcorn bag, making Teller Blume “famous for some months.” The U.S. state of Washington subsequently banned PFAS in food packaging, using the Coop Denmark’s popcorn bag as an inspiration. In 2016 Coop Denmark banned PFAS in outwear, textiles and home textiles. Two years later it prohibited PFAS in cleaning, cosmetics and personal care products, and in 2023 it took aim at PFAS outdoor textiles and garden furniture. In 2024 PFAS frying pans were banned. “I’ve been dedicated to [eliminating] PFAS since 2014 and besides raising my three children, this is the thing that I’m most proud of.” Malene Teller Blume, Coop Denmark Along with product bans, Coop Denmark has also contributed to national anti-PFAS legislation. It started a campaign in 2017 to ban the use of PFAS in paper and cardboard food contact materials (FCM). In September 2019 Denmark announced it would ban PFAS in FCM – the ban went into effect in July 2020 – making it the first country to do so. In addition, Coop Denmark works with organizations like ChemSec to advocate for PFAS bans at the EU level. Teller Blume shared a video explaining how Coop Denmark was able to persuade the Danish parliament to ban PFAS in food packaging. Early on, the company organized a social media campaign, backed by consumers and directed at members of parliament, sparking a debate on the problem of hazardous chemicals. Then, “together with experts, we prepared a complete post for a bill against hazardous chemicals, which could immediately be submitted into parliament,” the video said. “The campaign quickly gained the politicians attention; to ensure that no one missed this important message, we also surrounded the parliament building.” PFAS is not the only chemical contaminant that Coop Denmark has addressed over the course of its history, said Teller Blume; all told the company has taken 185 actions, including bans of PVC (polyvinyl chloride) in packaging in 1991, allergenic preservatives and fragrances in 1995 and bisphenol A in 2016. “We have tried to use early warnings, and also use the precautionary principle to set up requirements,” she said. “If there was a possible further solution, then we have put it in our trade agreements.” Teller Blume has met with leading anti-PFAS figures and environmental activists such as attorney Robert Bilott and scientist Arlene Blum. Years after he first met her, Bilott mentioned to Teller Blume that he has “told your story many times when people are saying that it’s not possible to face up to PFAS.”</t>
+          <t>A newly opened AstraZeneca pharmaceutical park in Qingdao, China, is equipped with a Haier Carrier CO2 (R744) heat pump system that provides comfort heating and cooling across the 54,000m2 (581,251ft2) complex.
+Haier Carrier shared the news in a press release detailing the project as well as a video posted to LinkedIn. The Qingdao site features both offices and R&amp;D facilities. The four dual-source HeatCO2OL heat pumps provide a heating capacity of 5.2MW (1,478TR) and a cooling capacity of 950kW (270TR). The heat pumps can provide simultaneous heating and cooling and offer “free heat recovery during cooling and waste heat reuse during heating.” The system also features 12 adiabatic gas coolers from BAC.
+The CO2 heat pumps are 40% more energy efficient than traditional fossil boilers, according to Haier Carrier. 
+BAC’s adiabatic coolers on the roof of AstraZeneca’s new pharmaceutical park in Qingdao, China. Photo credit: Haier Carrier
+Production milestone
+Haier Carrier also recently announced that it had completed China’s first automated production line for CO2 racks featuring a high-pressure explosion-proof test chamber. The automated production line will increase production eight-fold, the company said, while noting that the “first-of-its-kind testing chamber” meets stringent safety standards of 140bar (2,030psi) for CO2 systems.
+“From catching up in technology to independent innovation and from local manufacturing to global delivery, we are building a smart manufacturing base covering all commercial refrigeration and heating scenarios with digitalization, automation and greening as the core,” Haier Carrier said. “This production line is not just a production line but a declaration of China’s refrigeration and heating industry’s transformation toward green, intelligent and efficient development.”
+“This production line is not just a production line but a declaration of China’s refrigeration and heating industry’s transformation toward green, intelligent and efficient development.”
+Haier Carrier</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://naturalrefrigerants.com/news/atmo-europe-taking-a-stand-on-pfas/</t>
+          <t>https://naturalrefrigerants.com/news/haier-carrier-co2-heat-pump-provides-comfort-heating-and-cooling-for-new-astrazeneca-pharmaceutical-park-in-china/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Natural Refrigerants</t>
         </is>
       </c>
     </row>

</xml_diff>